<commit_message>
Dryer calculator: 1,750 Btu/lb confirmed for all drum types
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JENvqvx6kQMXayxjNDWASq
</commit_message>
<xml_diff>
--- a/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
+++ b/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="439">
   <si>
     <t xml:space="preserve">MCE DRYER HEAT &amp; MASS BALANCE CALCULATOR  ·  Rev A  ·  8 Sep 2026</t>
   </si>
@@ -141,7 +141,7 @@
     <t xml:space="preserve">Single-pass rotary drum</t>
   </si>
   <si>
-    <t xml:space="preserve">MCE standard</t>
+    <t xml:space="preserve">MCE standard, confirmed J. Shipley 9 Sep 2026</t>
   </si>
   <si>
     <t xml:space="preserve">MATERIAL AND THROUGHPUT</t>
@@ -150,9 +150,6 @@
     <t xml:space="preserve">Triple-pass rotary drum</t>
   </si>
   <si>
-    <t xml:space="preserve">MCE uses the same factor; confirm</t>
-  </si>
-  <si>
     <t xml:space="preserve">Wet feed rate</t>
   </si>
   <si>
@@ -163,9 +160,6 @@
   </si>
   <si>
     <t xml:space="preserve">Z8 eight-pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm</t>
   </si>
   <si>
     <t xml:space="preserve">Moisture in, wet basis</t>
@@ -2232,155 +2226,155 @@
         <v>1750</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>3000</v>
       </c>
       <c r="D7" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="G7" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>44</v>
       </c>
       <c r="H7" s="11" t="n">
         <v>1750</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>0.5</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H8" s="11" t="n">
         <v>1500</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>0.1</v>
       </c>
       <c r="D9" s="8"/>
       <c r="G9" s="8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H9" s="11" t="n">
         <v>1875</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>60</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>200</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C12" s="14" t="n">
         <v>0.35</v>
       </c>
       <c r="D12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="H12" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="I12" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="H12" s="15" t="s">
+      <c r="J12" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="I12" s="15" t="s">
+      <c r="K12" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="J12" s="15" t="s">
+      <c r="L12" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="K12" s="15" t="s">
+      <c r="M12" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="L12" s="15" t="s">
+      <c r="N12" s="15" t="s">
         <v>67</v>
-      </c>
-      <c r="M12" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="N12" s="15" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>8</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H13" s="12" t="n">
         <v>22800</v>
@@ -2401,21 +2395,21 @@
         <v>2.75</v>
       </c>
       <c r="N13" s="19" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>12</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H14" s="12" t="n">
         <v>19900</v>
@@ -2436,24 +2430,24 @@
         <v>3</v>
       </c>
       <c r="N14" s="19" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C15" s="12" t="n">
         <v>15</v>
       </c>
       <c r="D15" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="17" t="s">
         <v>78</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="17" t="s">
-        <v>80</v>
       </c>
       <c r="H15" s="12" t="n">
         <v>18500</v>
@@ -2474,18 +2468,18 @@
         <v>3.2</v>
       </c>
       <c r="N15" s="19" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="G16" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H16" s="12" t="n">
         <v>8500</v>
@@ -2506,21 +2500,21 @@
         <v>1.74</v>
       </c>
       <c r="N16" s="19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>1200</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H17" s="12" t="n">
         <v>8000</v>
@@ -2541,21 +2535,21 @@
         <v>1.74</v>
       </c>
       <c r="N17" s="19" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C18" s="9" t="n">
         <v>60</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H18" s="12" t="n">
         <v>12000</v>
@@ -2576,26 +2570,26 @@
         <v>2</v>
       </c>
       <c r="N18" s="19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C19" s="20" t="n">
         <v>0.01</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
@@ -2603,190 +2597,190 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>36</v>
       </c>
       <c r="D21" s="8"/>
       <c r="E21" s="10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C22" s="21" t="n">
         <f aca="false">INDEX($H$5:$H$9,MATCH(C21,$G$5:$G$9,0))</f>
         <v>1750</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D23" s="8"/>
       <c r="E23" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C24" s="21" t="n">
         <f aca="false">INDEX($H$13:$H$18,MATCH(C23,$G$13:$G$18,0))</f>
         <v>22800</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C25" s="22" t="n">
         <f aca="false">INDEX($J$13:$J$18,MATCH(C23,$G$13:$G$18,0))</f>
         <v>0.25</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">INDEX($K$13:$K$18,MATCH(C23,$G$13:$G$18,0))</f>
         <v>16.33</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">INDEX($L$13:$L$18,MATCH(C23,$G$13:$G$18,0))</f>
         <v>2.25</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C28" s="23" t="n">
         <f aca="false">INDEX($M$13:$M$18,MATCH(C23,$G$13:$G$18,0))</f>
         <v>2.75</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C29" s="12" t="n">
         <v>600</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C30" s="12" t="n">
         <v>180</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C31" s="18" t="n">
         <v>0.9</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C32" s="18" t="n">
         <v>0.03</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C33" s="18" t="n">
         <v>0.1</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C34" s="14" t="n">
         <v>8</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
@@ -2794,124 +2788,124 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C36" s="12" t="n">
         <v>350</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C37" s="16" t="n">
         <v>10</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C38" s="18" t="n">
         <v>0.65</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C39" s="12" t="n">
         <v>5000</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C40" s="12" t="n">
         <v>3300</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C41" s="16" t="n">
         <v>3</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C42" s="18" t="n">
         <v>0.2</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C43" s="18" t="n">
         <v>0.15</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C44" s="12" t="n">
         <v>1200</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C45" s="6"/>
       <c r="D45" s="6"/>
@@ -2919,36 +2913,36 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C46" s="12" t="n">
         <v>24</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="8" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C47" s="12" t="n">
         <v>312</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C48" s="21" t="n">
         <f aca="false">C46*C47</f>
         <v>7488</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -2989,12 +2983,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -3002,106 +2996,106 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C4" s="24" t="n">
         <f aca="false">Inputs!$C$7</f>
         <v>3000</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C5" s="21" t="n">
         <f aca="false">Inputs!$C$7*(1-Inputs!$C$8)</f>
         <v>1500</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C6" s="21" t="n">
         <f aca="false">Inputs!$C$7*Inputs!$C$8</f>
         <v>1500</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="7" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C7" s="25" t="n">
         <f aca="false">HMB!$C$5/(1-Inputs!$C$9)</f>
         <v>1666.66666666667</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C8" s="21" t="n">
         <f aca="false">HMB!$C$7-HMB!$C$5</f>
         <v>166.666666666667</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">HMB!$C$6-HMB!$C$8</f>
         <v>1333.33333333333</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C10" s="26" t="n">
         <f aca="false">HMB!$C$9/8.345</f>
         <v>159.776313161574</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C11" s="23" t="n">
         <f aca="false">HMB!$C$7/2000</f>
         <v>0.833333333333333</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -3109,61 +3103,61 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C13" s="26" t="n">
         <f aca="false">1.01*(212-Inputs!$C$10)+970.4</f>
         <v>1123.92</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C14" s="24" t="n">
         <f aca="false">Inputs!$C$22</f>
         <v>1750</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C15" s="25" t="n">
         <f aca="false">HMB!$C$9*HMB!$C$14</f>
         <v>2333333.33333333</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C16" s="23" t="n">
         <f aca="false">HMB!$C$15/1000000</f>
         <v>2.33333333333333</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
@@ -3171,136 +3165,136 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C18" s="21" t="n">
         <f aca="false">HMB!$C$5*Inputs!$C$12*(Inputs!$C$11-Inputs!$C$10)</f>
         <v>73500</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C19" s="21" t="n">
         <f aca="false">HMB!$C$8*1*(Inputs!$C$11-Inputs!$C$10)</f>
         <v>23333.3333333333</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C20" s="21" t="n">
         <f aca="false">HMB!$C$9*1.01*(212-Inputs!$C$10)</f>
         <v>204693.333333333</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C21" s="21" t="n">
         <f aca="false">HMB!$C$9*970.4</f>
         <v>1293866.66666667</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C22" s="21" t="n">
         <f aca="false">HMB!$C$9*0.45*(Inputs!$C$30-212)</f>
         <v>-19200</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C23" s="25" t="n">
         <f aca="false">SUM($C$18:$C$22)</f>
         <v>1576193.33333333</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C24" s="27" t="n">
         <f aca="false">Inputs!$C$31*(Inputs!$C$29-Inputs!$C$30)/(Inputs!$C$29-Inputs!$C$18)</f>
         <v>0.7</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C25" s="25" t="n">
         <f aca="false">HMB!$C$23/(HMB!$C$24-Inputs!$C$32)</f>
         <v>2352527.36318408</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">HMB!$C$25/1000000</f>
         <v>2.35252736318408</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C27" s="25" t="n">
         <f aca="false">HMB!$C$25/HMB!$C$9</f>
         <v>1764.39552238806</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C28" s="21" t="str">
         <f aca="false">IF(ABS(HMB!$C$27/HMB!$C$14-1)&lt;=0.15,"WITHIN 15% OF MCE FACTOR",IF(HMB!$C$27&gt;HMB!$C$14,"RIGOROUS IS HIGHER: raise inlet temp or accept higher fuel","RIGOROUS IS LOWER: MCE factor is conservative here"))</f>
@@ -3308,27 +3302,27 @@
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C29" s="25" t="n">
         <f aca="false">MAX(HMB!$C$15,HMB!$C$25)</f>
         <v>2352527.36318408</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
@@ -3336,85 +3330,85 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C31" s="28" t="n">
         <f aca="false">HMB!$C$29/Inputs!$C$24</f>
         <v>103.181024701056</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C32" s="26" t="n">
         <f aca="false">HMB!$C$31/INDEX(Inputs!$I$13:$I$18,MATCH(Inputs!$C$23,Inputs!$G$13:$G$18,0))/60</f>
         <v>39.0837214776728</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="8" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C33" s="21" t="n">
         <f aca="false">HMB!$C$31*Inputs!$C$26*(1+Inputs!$C$25)</f>
         <v>2106.18266671031</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C34" s="21" t="n">
         <f aca="false">HMB!$C$31+HMB!$C$33</f>
         <v>2209.36369141136</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C35" s="21" t="n">
         <f aca="false">HMB!$C$31*Inputs!$C$27+HMB!$C$33*Inputs!$C$19</f>
         <v>253.219132244479</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C36" s="21" t="n">
         <f aca="false">Inputs!$C$18+HMB!$C$29*Inputs!$C$31/(0.27*HMB!$C$34)</f>
         <v>3609.32866316404</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="5" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
@@ -3422,37 +3416,37 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C38" s="25" t="n">
         <f aca="false">HMB!$C$29*Inputs!$C$31/(0.24*(Inputs!$C$29-Inputs!$C$18))</f>
         <v>16336.9955776672</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C39" s="21" t="n">
         <f aca="false">HMB!$C$38-HMB!$C$34</f>
         <v>14127.6318862559</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C40" s="21" t="str">
         <f aca="false">IF(HMB!$C$39&lt;0,"INLET TEMP TOO HIGH FOR THIS FUEL / EXCESS AIR","OK")</f>
@@ -3462,67 +3456,67 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="8" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C41" s="21" t="n">
         <f aca="false">HMB!$C$38*Inputs!$C$33</f>
         <v>1633.69955776672</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="C42" s="21" t="n">
         <f aca="false">HMB!$C$38+HMB!$C$41</f>
         <v>17970.6951354339</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C43" s="21" t="n">
         <f aca="false">HMB!$C$35+(HMB!$C$39+HMB!$C$41)*Inputs!$C$19+HMB!$C$9</f>
         <v>1744.16578001804</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C44" s="25" t="n">
         <f aca="false">HMB!$C$42+HMB!$C$43</f>
         <v>19714.860915452</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C45" s="27" t="n">
         <f aca="false">HMB!$C$43/HMB!$C$42</f>
         <v>0.097056110900182</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="8" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C46" s="29" t="n">
         <f aca="false">(1-0.0000068754*Inputs!$C$17)^5.2559</f>
@@ -3530,90 +3524,90 @@
       </c>
       <c r="D46" s="8"/>
       <c r="E46" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="8" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C47" s="29" t="n">
         <f aca="false">0.0765*530/(460+Inputs!$C$30)*HMB!$C$46</f>
         <v>0.0606522054005384</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C48" s="29" t="n">
         <f aca="false">0.0476*530/(460+Inputs!$C$30)*HMB!$C$46</f>
         <v>0.0377391500270017</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C49" s="25" t="n">
         <f aca="false">HMB!$C$42/HMB!$C$47/60+HMB!$C$43/HMB!$C$48/60</f>
         <v>5708.45379083241</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C50" s="21" t="n">
         <f aca="false">HMB!$C$42/0.075/60+HMB!$C$43/0.0467/60</f>
         <v>4615.95953521827</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C51" s="21" t="n">
         <f aca="false">(HMB!$C$38/(0.0765*530/(460+Inputs!$C$29)*HMB!$C$46)+HMB!$C$35/(0.0476*530/(460+Inputs!$C$29)*HMB!$C$46))/60</f>
         <v>7620.54600641747</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C52" s="26" t="n">
         <f aca="false">HMB!$C$42/HMB!$C$7</f>
         <v>10.7824170812604</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C53" s="21" t="str">
         <f aca="false">IF(HMB!$C$52&gt;=Inputs!$C$41,"CONVEYING CAN OCCUR","CONVEYING CANNOT OCCUR: add recycle or raise airflow")</f>
@@ -3623,7 +3617,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="5" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="6"/>
@@ -3631,85 +3625,85 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="8" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C55" s="21" t="n">
         <f aca="false">HMB!$C$29</f>
         <v>2352527.36318408</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C56" s="21" t="n">
         <f aca="false">HMB!$C$29*(1-Inputs!$C$31)</f>
         <v>235252.736318408</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="8" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C57" s="21" t="n">
         <f aca="false">HMB!$C$23*HMB!$C$29/HMB!$C$25</f>
         <v>1576193.33333333</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="8" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C58" s="21" t="n">
         <f aca="false">HMB!$C$29*Inputs!$C$32</f>
         <v>70575.8208955224</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C59" s="21" t="n">
         <f aca="false">HMB!$C$38*0.24*(Inputs!$C$30-Inputs!$C$18)</f>
         <v>470505.472636816</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="7" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C60" s="25" t="n">
         <f aca="false">HMB!$C$55-HMB!$C$56-HMB!$C$57-HMB!$C$58-HMB!$C$59</f>
         <v>0</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C61" s="30" t="n">
         <f aca="false">HMB!$C$60/HMB!$C$55</f>
@@ -3719,7 +3713,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="6"/>
@@ -3727,7 +3721,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="8" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C63" s="24" t="str">
         <f aca="false">Equipment!$C$4</f>
@@ -3737,56 +3731,56 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C64" s="24" t="n">
         <f aca="false">Equipment!$C$7</f>
         <v>589.048622548086</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C65" s="31" t="n">
         <f aca="false">IF(HMB!$C$64&gt;0,HMB!$C$9/HMB!$C$64,"n/a")</f>
         <v>2.26353696841807</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="8" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C66" s="26" t="n">
         <f aca="false">Inputs!$C$7/60*Inputs!$C$15/Inputs!$C$14</f>
         <v>62.5</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C67" s="30" t="n">
         <f aca="false">IF(HMB!$C$64&gt;0,HMB!$C$66/HMB!$C$64,"n/a")</f>
         <v>0.106103295394597</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -3823,27 +3817,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="K2" s="32" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="L2" s="33" t="n">
         <v>6</v>
       </c>
       <c r="M2" s="32" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="N2" s="33" t="n">
         <v>8</v>
       </c>
       <c r="O2" s="32" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="P2" s="33" t="n">
         <v>8</v>
@@ -3851,54 +3845,54 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>252</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="E5" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="F5" s="15" t="s">
         <v>254</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="G5" s="15" t="s">
         <v>255</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="H5" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="I5" s="15" t="s">
         <v>257</v>
       </c>
-      <c r="H5" s="15" t="s">
+      <c r="J5" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="I5" s="15" t="s">
+      <c r="K5" s="15" t="s">
         <v>259</v>
       </c>
-      <c r="J5" s="15" t="s">
+      <c r="L5" s="15" t="s">
         <v>260</v>
       </c>
-      <c r="K5" s="15" t="s">
+      <c r="M5" s="15" t="s">
         <v>261</v>
       </c>
-      <c r="L5" s="15" t="s">
+      <c r="N5" s="15" t="s">
         <v>262</v>
       </c>
-      <c r="M5" s="15" t="s">
+      <c r="O5" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="N5" s="15" t="s">
+      <c r="P5" s="15" t="s">
         <v>264</v>
-      </c>
-      <c r="O5" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="P5" s="15" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3906,7 +3900,7 @@
         <v>36</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>3</v>
@@ -3946,11 +3940,11 @@
         <v>99999</v>
       </c>
       <c r="N6" s="36" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="O6" s="37"/>
       <c r="P6" s="10" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3958,7 +3952,7 @@
         <v>36</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D7" s="9" t="n">
         <v>5</v>
@@ -3998,7 +3992,7 @@
       <c r="N7" s="36"/>
       <c r="O7" s="37"/>
       <c r="P7" s="10" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4006,7 +4000,7 @@
         <v>36</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D8" s="9" t="n">
         <v>6</v>
@@ -4048,7 +4042,7 @@
       <c r="N8" s="36"/>
       <c r="O8" s="37"/>
       <c r="P8" s="10" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4056,7 +4050,7 @@
         <v>36</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>8</v>
@@ -4096,11 +4090,11 @@
         <v>9</v>
       </c>
       <c r="N9" s="36" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="O9" s="37"/>
       <c r="P9" s="10" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4108,7 +4102,7 @@
         <v>39</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D10" s="39"/>
       <c r="E10" s="39"/>
@@ -4141,7 +4135,7 @@
       <c r="N10" s="36"/>
       <c r="O10" s="37"/>
       <c r="P10" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4149,7 +4143,7 @@
         <v>39</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D11" s="39"/>
       <c r="E11" s="39"/>
@@ -4182,7 +4176,7 @@
       <c r="N11" s="36"/>
       <c r="O11" s="37"/>
       <c r="P11" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4190,7 +4184,7 @@
         <v>39</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D12" s="39"/>
       <c r="E12" s="39"/>
@@ -4223,7 +4217,7 @@
       <c r="N12" s="36"/>
       <c r="O12" s="37"/>
       <c r="P12" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4231,7 +4225,7 @@
         <v>39</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D13" s="39"/>
       <c r="E13" s="39"/>
@@ -4264,15 +4258,15 @@
       <c r="N13" s="36"/>
       <c r="O13" s="37"/>
       <c r="P13" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="D14" s="9" t="n">
         <v>6</v>
@@ -4311,15 +4305,15 @@
       <c r="N14" s="36"/>
       <c r="O14" s="37"/>
       <c r="P14" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D15" s="9" t="n">
         <v>8</v>
@@ -4358,15 +4352,15 @@
       <c r="N15" s="36"/>
       <c r="O15" s="37"/>
       <c r="P15" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="D16" s="9" t="n">
         <v>10</v>
@@ -4405,15 +4399,15 @@
       <c r="N16" s="36"/>
       <c r="O16" s="37"/>
       <c r="P16" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D17" s="9" t="n">
         <v>10</v>
@@ -4452,15 +4446,15 @@
       <c r="N17" s="36"/>
       <c r="O17" s="37"/>
       <c r="P17" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D18" s="9" t="n">
         <v>12</v>
@@ -4499,15 +4493,15 @@
       <c r="N18" s="36"/>
       <c r="O18" s="37"/>
       <c r="P18" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D19" s="9" t="n">
         <v>12</v>
@@ -4546,15 +4540,15 @@
       <c r="N19" s="36"/>
       <c r="O19" s="37"/>
       <c r="P19" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>12</v>
@@ -4593,15 +4587,15 @@
       <c r="N20" s="36"/>
       <c r="O20" s="37"/>
       <c r="P20" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>13</v>
@@ -4640,15 +4634,15 @@
       <c r="N21" s="36"/>
       <c r="O21" s="37"/>
       <c r="P21" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D22" s="9" t="n">
         <v>14</v>
@@ -4687,15 +4681,15 @@
       <c r="N22" s="36"/>
       <c r="O22" s="37"/>
       <c r="P22" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>15</v>
@@ -4734,7 +4728,7 @@
       <c r="N23" s="36"/>
       <c r="O23" s="37"/>
       <c r="P23" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -4765,12 +4759,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -4778,7 +4772,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C4" s="25" t="str">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$C$6:$C$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0)),"NO MODEL OF THIS TYPE MEETS THE JOB - fill ratings or pick another type")</f>
@@ -4788,79 +4782,79 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C5" s="26" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$D$6:$D$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0)),"")</f>
         <v>5</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C6" s="26" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$E$6:$E$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0)),"")</f>
         <v>30</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C7" s="21" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$G$6:$G$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0)),0)</f>
         <v>589.048622548086</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C8" s="21" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$H$6:$H$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0)),"")</f>
         <v>6872.23392972767</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C9" s="21" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$L$6:$L$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0)),"")</f>
         <v>3534.29173528852</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C10" s="26" t="str">
         <f aca="false">IFERROR(IF(INDEX('Dryer Models'!$I$6:$I$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0))="","not entered",INDEX('Dryer Models'!$I$6:$I$23,MATCH(MIN('Dryer Models'!$M$6:$M$23),'Dryer Models'!$M$6:$M$23,0))),"")</f>
         <v>not entered</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C11" s="22" t="n">
         <f aca="false">IF(ISNUMBER(Equipment!$C$8),HMB!$C$49/Equipment!$C$8,"")</f>
@@ -4870,7 +4864,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">IF(ISNUMBER(Equipment!$C$9),HMB!$C$9/Equipment!$C$9,"")</f>
@@ -4880,7 +4874,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="5" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
@@ -4888,31 +4882,31 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C14" s="41" t="n">
         <f aca="false">HMB!$C$29/1000000</f>
         <v>2.35252736318408</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C15" s="31" t="n">
         <f aca="false">Equipment!$C$14*(1+Inputs!$C$42)</f>
         <v>2.8230328358209</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C16" s="21" t="str">
         <f aca="false">IF(AND(ISNUMBER(Equipment!$C$10),Equipment!$C$10&gt;0),IF(Equipment!$C$15&lt;=Equipment!$C$10,"WITHIN MODEL BURNER RATING","EXCEEDS MODEL BURNER RATING - next size or bigger burner"),"model burner rating not entered")</f>
@@ -4922,46 +4916,46 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="C17" s="21" t="n">
         <f aca="false">Equipment!$C$15*1000000/Inputs!$C$44</f>
         <v>2352.52736318408</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C18" s="26" t="n">
         <f aca="false">Equipment!$C$17/576</f>
         <v>4.08424889441681</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C19" s="26" t="n">
         <f aca="false">Equipment!$C$17/135</f>
         <v>17.4261286161784</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="C20" s="21" t="n">
         <f aca="false">ROUNDUP(Equipment!$C$15*100,-1)</f>
@@ -4969,12 +4963,12 @@
       </c>
       <c r="D20" s="8"/>
       <c r="E20" s="10" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -4982,139 +4976,139 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">HMB!$C$49</f>
         <v>5708.45379083241</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C23" s="24" t="n">
         <f aca="false">Inputs!$C$30</f>
         <v>180</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C24" s="26" t="n">
         <f aca="false">Equipment!$C$22*Inputs!$C$37/(6356*Inputs!$C$38)</f>
         <v>13.8172382021407</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="7" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C25" s="25" t="n">
         <f aca="false">INDEX(Tables!$B$4:$B$21,COUNTIF(Tables!$B$4:$B$21,"&lt;"&amp;Equipment!$C$24*1.15)+1)</f>
         <v>20</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C26" s="26" t="n">
         <f aca="false">SQRT(Equipment!$C$22/Inputs!$C$39*4/PI())*12</f>
         <v>14.4680682278768</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C27" s="25" t="n">
         <f aca="false">CEILING(Equipment!$C$26,2)</f>
         <v>16</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C28" s="21" t="n">
         <f aca="false">Equipment!$C$22/(PI()/4*(Equipment!$C$27/12)^2)</f>
         <v>4088.37887200191</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="8" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C29" s="21" t="n">
         <f aca="false">CEILING(SQRT(HMB!$C$51/Inputs!$C$39*4/PI())*12,2)</f>
         <v>18</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C30" s="21" t="n">
         <f aca="false">Equipment!$C$22/Inputs!$C$40*144</f>
         <v>249.096165418141</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="8" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C31" s="21" t="n">
         <f aca="false">SQRT(Equipment!$C$22/Inputs!$C$40/0.125)*12</f>
         <v>44.6404449277237</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
@@ -5122,31 +5116,31 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="8" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C33" s="23" t="n">
         <f aca="false">HMB!$C$7/Inputs!$C$13/60</f>
         <v>3.47222222222222</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="8" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C34" s="23" t="n">
         <f aca="false">Inputs!$C$7/Inputs!$C$14/60</f>
         <v>4.16666666666667</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="7" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C35" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Tables!$E$4:$E$13,COUNTIF(Tables!$H$4:$H$13,"&lt;"&amp;Equipment!$C$33)+1),"none in table")</f>
@@ -5156,7 +5150,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C36" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Tables!$E$4:$E$13,COUNTIF(Tables!$H$4:$H$13,"&lt;"&amp;Equipment!$C$34)+1),"none in table")</f>
@@ -5166,19 +5160,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="8" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C37" s="21" t="n">
         <f aca="false">IFERROR(INDEX(Tables!$J$4:$J$13,COUNTIF(Tables!$M$4:$M$13,"&lt;"&amp;Equipment!$C$34*60)+1),"none in table")</f>
         <v>9</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="5" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
@@ -5186,86 +5180,86 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C39" s="24" t="n">
         <f aca="false">Inputs!$C$48</f>
         <v>7488</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C40" s="21" t="n">
         <f aca="false">HMB!$C$7*Equipment!$C$39/2000</f>
         <v>6240</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="8" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C41" s="21" t="n">
         <f aca="false">HMB!$C$9*Equipment!$C$39/2000</f>
         <v>4992</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C42" s="21" t="n">
         <f aca="false">HMB!$C$31*Equipment!$C$39/2000</f>
         <v>386.309756480754</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C43" s="21" t="n">
         <f aca="false">HMB!$C$29*Equipment!$C$39/1000000</f>
         <v>17615.7248955224</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C44" s="42" t="n">
         <f aca="false">Equipment!$C$43*Inputs!$C$34</f>
         <v>140925.799164179</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="7" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C45" s="43" t="n">
         <f aca="false">IF(Equipment!$C$40&gt;0,Equipment!$C$44/Equipment!$C$40,0)</f>
         <v>22.5842626865672</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -5302,39 +5296,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>349</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="G3" s="15" t="s">
         <v>350</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="H3" s="15" t="s">
         <v>351</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="I3" s="15" t="s">
         <v>352</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="J3" s="15" t="s">
         <v>353</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="K3" s="15" t="s">
         <v>354</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="L3" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="M3" s="15" t="s">
         <v>355</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>356</v>
-      </c>
-      <c r="L3" s="15" t="s">
-        <v>352</v>
-      </c>
-      <c r="M3" s="15" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5652,10 +5646,10 @@
         <v>75</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5723,12 +5717,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -5739,119 +5733,119 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C4" s="14" t="n">
         <v>0.1</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C5" s="14" t="n">
         <v>0.08</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C6" s="46" t="n">
         <v>0.0006</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C7" s="14" t="n">
         <v>0.9</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C8" s="14" t="n">
         <v>3</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>0.9</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>0.7</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>0.15</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="5" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -5862,27 +5856,27 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="15" t="s">
+        <v>379</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>380</v>
+      </c>
+      <c r="E13" s="15" t="s">
         <v>381</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D13" s="15" t="s">
+      <c r="F13" s="15" t="s">
         <v>382</v>
       </c>
-      <c r="E13" s="15" t="s">
-        <v>383</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>384</v>
-      </c>
       <c r="G13" s="15" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="C14" s="47" t="n">
         <f aca="false">HMB!$C$31*Inputs!$C$28</f>
@@ -5907,7 +5901,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C15" s="47" t="n">
         <f aca="false">HMB!$C$29/1000000*Emissions!$C$4</f>
@@ -5932,7 +5926,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="C16" s="47" t="n">
         <f aca="false">HMB!$C$29/1000000*Emissions!$C$5</f>
@@ -5957,7 +5951,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C17" s="47" t="n">
         <f aca="false">HMB!$C$29/1000000*Emissions!$C$6</f>
@@ -5982,7 +5976,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="C18" s="47" t="n">
         <f aca="false">Emissions!$C$7*(HMB!$C$5/2000)</f>
@@ -6007,7 +6001,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C19" s="47" t="n">
         <f aca="false">Emissions!$C$11*Emissions!$C$7*(HMB!$C$5/2000)</f>
@@ -6032,7 +6026,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="C20" s="47" t="n">
         <f aca="false">Emissions!$C$8*(HMB!$C$5/2000)*(1-Emissions!$C$9)</f>
@@ -6057,7 +6051,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C21" s="47" t="n">
         <f aca="false">Emissions!$C$8*(HMB!$C$5/2000)*(1-Emissions!$C$9)*Emissions!$C$10</f>
@@ -6108,12 +6102,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -6121,55 +6115,55 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C4" s="24" t="n">
         <f aca="false">Inputs!$C$7/2.20462</f>
         <v>1360.77872830692</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C5" s="50" t="n">
         <f aca="false">Inputs!$C$7/2.20462/1000</f>
         <v>1.36077872830692</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">HMB!$C$7/2.20462</f>
         <v>755.988182392733</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">HMB!$C$9/2.20462</f>
         <v>604.790545914186</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C8" s="51" t="str">
         <f aca="false">TEXT(Inputs!$C$8,"0.0%")&amp;" / "&amp;TEXT(Inputs!$C$9,"0.0%")</f>
@@ -6179,7 +6173,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="5" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -6187,79 +6181,79 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">HMB!$C$13*2.326</f>
         <v>2614.23792</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C11" s="24" t="n">
         <f aca="false">HMB!$C$14*2.326</f>
         <v>4070.5</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C12" s="50" t="n">
         <f aca="false">HMB!$C$29*1.05506/1000000</f>
         <v>2.482057519801</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C13" s="24" t="n">
         <f aca="false">HMB!$C$29*0.293071/1000</f>
         <v>689.457546855722</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C14" s="51" t="n">
         <f aca="false">HMB!$C$31/2.20462</f>
         <v>46.8021811927027</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">Inputs!$C$24*2.326</f>
         <v>53032.8</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="5" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -6267,31 +6261,31 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C17" s="51" t="str">
         <f aca="false">TEXT((Inputs!$C$10-32)*5/9,"0")&amp;" / "&amp;TEXT((Inputs!$C$11-32)*5/9,"0")</f>
         <v>16 / 93</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C18" s="51" t="str">
         <f aca="false">TEXT((Inputs!$C$29-32)*5/9,"0")&amp;" / "&amp;TEXT((Inputs!$C$30-32)*5/9,"0")</f>
         <v>316 / 82</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="5" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -6299,55 +6293,55 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">HMB!$C$38/2.20462</f>
         <v>7410.34535551126</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C21" s="24" t="n">
         <f aca="false">HMB!$C$44/2.20462</f>
         <v>8942.52112175885</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">HMB!$C$49*1.69901</f>
         <v>9698.72007516217</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C23" s="24" t="n">
         <f aca="false">HMB!$C$50*1.69901*273.15/294.26</f>
         <v>7279.94171522702</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="5" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
@@ -6355,7 +6349,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="8" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C25" s="51" t="str">
         <f aca="false">Equipment!$C$4</f>
@@ -6365,62 +6359,62 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="C26" s="51" t="str">
         <f aca="false">IF(ISNUMBER(Equipment!$C$5),TEXT(Equipment!$C$5*0.3048,"0.00")&amp;" × "&amp;TEXT(Equipment!$C$6*0.3048,"0.0"),"")</f>
         <v>1.52 × 9.1</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C27" s="41" t="n">
         <f aca="false">Equipment!$C$15*0.293071</f>
         <v>0.827349056226866</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C28" s="51" t="n">
         <f aca="false">Equipment!$C$25*0.7457</f>
         <v>14.914</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="8" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C29" s="24" t="n">
         <f aca="false">Equipment!$C$27*25.4</f>
         <v>406.4</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C30" s="24" t="n">
         <f aca="false">Inputs!$C$37*249.09</f>
         <v>2490.9</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -6449,24 +6443,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="15" t="s">
+        <v>419</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>421</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="E3" s="15" t="s">
         <v>422</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="F3" s="15" t="s">
         <v>423</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>424</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6477,18 +6471,18 @@
         <v>35</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>426</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>427</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="52" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C5" s="9" t="n">
         <v>3000</v>
@@ -6505,7 +6499,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="52" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C6" s="18" t="n">
         <v>0.5</v>
@@ -6522,7 +6516,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="52" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C7" s="18" t="n">
         <v>0.1</v>
@@ -6539,7 +6533,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="52" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C8" s="9" t="n">
         <v>60</v>
@@ -6556,7 +6550,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="52" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>200</v>
@@ -6573,7 +6567,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="52" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>600</v>
@@ -6590,7 +6584,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="52" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>180</v>
@@ -6607,7 +6601,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="52" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>1750</v>
@@ -6624,19 +6618,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="52" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6644,16 +6638,16 @@
         <v>30</v>
       </c>
       <c r="C14" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="F14" s="9" t="s">
         <v>438</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>439</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dryer calculator Rev D: live Flow sheet, reactor defaults confirmed, triple-pass to match Baker-Rullman
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JENvqvx6kQMXayxjNDWASq
</commit_message>
<xml_diff>
--- a/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
+++ b/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
@@ -1255,7 +1255,7 @@
     <t xml:space="preserve">TP-36 (3'×12')</t>
   </si>
   <si>
-    <t xml:space="preserve">Same shell sizes as single-pass; ACFM = OD cross-section × face velocity × triple-pass factor until Baker-Rullman ratings are entered</t>
+    <t xml:space="preserve">MCE will match the Baker-Rullman triple-pass models; ACFM = OD cross-section × face velocity × triple-pass factor until their ratings are entered</t>
   </si>
   <si>
     <t xml:space="preserve">TP-36 (3'×20')</t>
@@ -1648,7 +1648,7 @@
     <t xml:space="preserve">fraction of dry feed</t>
   </si>
   <si>
-    <t xml:space="preserve">See table at right; Prozus report assumed 1.0, which is why its 67% product was wrong</t>
+    <t xml:space="preserve">MCE default, confirmed J. Shipley 9 Sep 2026. See table at right; Prozus report assumed 1.0, which is why its 67% product was wrong</t>
   </si>
   <si>
     <t xml:space="preserve">Char heating value</t>
@@ -1666,7 +1666,7 @@
     <t xml:space="preserve">Btu/lb dry feed</t>
   </si>
   <si>
-    <t xml:space="preserve">+ endothermic; wood slow pyrolysis roughly 0 to +200</t>
+    <t xml:space="preserve">MCE default, confirmed J. Shipley 9 Sep 2026; + endothermic, wood slow pyrolysis roughly 0 to +200</t>
   </si>
   <si>
     <t xml:space="preserve">Specific heat, dry feed</t>
@@ -1726,7 +1726,7 @@
     <t xml:space="preserve">Btu/hr·ft²</t>
   </si>
   <si>
-    <t xml:space="preserve">Indirect rotary reactors 2,000–6,000; confirm with MCE shell design</t>
+    <t xml:space="preserve">MCE default, confirmed J. Shipley 9 Sep 2026; indirect rotary reactors 2,000–6,000</t>
   </si>
   <si>
     <t xml:space="preserve">Feed, wet</t>

</xml_diff>

<commit_message>
Dryer calculator Rev E: brochure renders on the Flow sheet, case runner, LETEK 140 MT/day run and PFD
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JENvqvx6kQMXayxjNDWASq
</commit_message>
<xml_diff>
--- a/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
+++ b/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
@@ -1968,7 +1968,7 @@
     <numFmt numFmtId="173" formatCode="0.000"/>
     <numFmt numFmtId="174" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2106,20 +2106,6 @@
     <font>
       <b val="true"/>
       <sz val="13"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -2687,6 +2673,117 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>1440</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>209160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7627680" y="3390840"/>
+          <a:ext cx="4161960" cy="1676160"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>57</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>61</xdr:col>
+      <xdr:colOff>84960</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>209160</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13174920" y="2971800"/>
+          <a:ext cx="1009440" cy="3142800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>43</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>50</xdr:col>
+      <xdr:colOff>19800</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>66240</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9938880" y="666720"/>
+          <a:ext cx="1638000" cy="1323720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
@@ -2702,7 +2799,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="1" name="shape301"/>
+        <xdr:cNvPr id="4" name="shape301"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2747,7 +2844,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="shape302"/>
+        <xdr:cNvPr id="5" name="shape302"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -2816,7 +2913,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="3" name="line303"/>
+        <xdr:cNvPr id="6" name="line303"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -2852,7 +2949,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="4" name="line304"/>
+        <xdr:cNvPr id="7" name="line304"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -2889,7 +2986,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="5" name="line305"/>
+        <xdr:cNvPr id="8" name="line305"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -2925,7 +3022,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="6" name="line306"/>
+        <xdr:cNvPr id="9" name="line306"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -2955,20 +3052,20 @@
       <xdr:rowOff>167400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>231120</xdr:colOff>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>43920</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>167400</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="7" name="line307"/>
+        <xdr:cNvPr id="10" name="line307"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4160520" y="4396680"/>
-          <a:ext cx="3236400" cy="360"/>
+          <a:ext cx="3511440" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -2999,7 +3096,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="8" name="line308"/>
+        <xdr:cNvPr id="11" name="line308"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -3036,7 +3133,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="9" name="line309"/>
+        <xdr:cNvPr id="12" name="line309"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -3073,7 +3170,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="10" name="line310"/>
+        <xdr:cNvPr id="13" name="line310"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -3102,20 +3199,20 @@
       <xdr:rowOff>41760</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>231120</xdr:colOff>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>43920</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>41760</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="11" name="line311"/>
+        <xdr:cNvPr id="14" name="line311"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6472080" y="4690080"/>
-          <a:ext cx="924840" cy="360"/>
+          <a:ext cx="1199880" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3133,347 +3230,8 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="shape312"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7396560" y="3935520"/>
-          <a:ext cx="230760" cy="838080"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="shape313"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7627680" y="3726000"/>
-          <a:ext cx="230760" cy="1257120"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="shape314"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8089920" y="3726000"/>
-          <a:ext cx="230760" cy="1257120"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>47</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="shape315"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8321040" y="3516480"/>
-          <a:ext cx="2773440" cy="1676160"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr lIns="0" rIns="0" tIns="45000" bIns="45000" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="1" lang="en-US" sz="1400" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-            </a:rPr>
-            <a:t>XD Series Rotary Dryer</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1400" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>48</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>48</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="16" name="shape316"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11094840" y="3726000"/>
-          <a:ext cx="230760" cy="1257120"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>50</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>50</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="17" name="shape317"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11557080" y="3726000"/>
-          <a:ext cx="230760" cy="1257120"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
       <xdr:col>51</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>51</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="18" name="shape318"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="11788200" y="3935520"/>
-          <a:ext cx="230760" cy="838080"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ededdf"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>52</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>132480</xdr:colOff>
       <xdr:row>20</xdr:row>
       <xdr:rowOff>125640</xdr:rowOff>
     </xdr:from>
@@ -3485,13 +3243,13 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="19" name="line319"/>
+        <xdr:cNvPr id="15" name="line312"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12019320" y="4354920"/>
-          <a:ext cx="693720" cy="360"/>
+          <a:off x="11920680" y="4354920"/>
+          <a:ext cx="792360" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3511,7 +3269,7 @@
       <xdr:col>55</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>167400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>55</xdr:col>
@@ -3521,13 +3279,13 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="20" name="line320"/>
+        <xdr:cNvPr id="16" name="line313"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="12712680" y="3642120"/>
-          <a:ext cx="360" cy="713160"/>
+          <a:off x="12712680" y="3767760"/>
+          <a:ext cx="360" cy="587520"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3547,23 +3305,23 @@
       <xdr:col>55</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>167400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>56</xdr:col>
-      <xdr:colOff>231120</xdr:colOff>
+      <xdr:col>57</xdr:col>
+      <xdr:colOff>132480</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
+      <xdr:rowOff>167400</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="21" name="line321"/>
+        <xdr:cNvPr id="17" name="line314"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12712680" y="3642120"/>
-          <a:ext cx="462600" cy="360"/>
+          <a:off x="12712680" y="3767760"/>
+          <a:ext cx="595080" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3581,232 +3339,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>57</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>41760</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>57</xdr:col>
-      <xdr:colOff>230760</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>83160</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="shape322"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="13174920" y="3432600"/>
-          <a:ext cx="230760" cy="460440"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="dce6f1"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>58</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>62</xdr:col>
-      <xdr:colOff>231120</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>209160</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="shape323"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="13406040" y="3181320"/>
-          <a:ext cx="1155600" cy="1257120"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="dce6f1"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr lIns="0" rIns="0" tIns="90000" bIns="90000" anchor="ctr" vert="vert270">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="1" lang="en-US" sz="1200" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-            </a:rPr>
-            <a:t>Cyclone Collector</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1200" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>58</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>-360</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>62</xdr:col>
-      <xdr:colOff>231120</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>208800</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="shape324"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm flipV="1">
-          <a:off x="13406040" y="4438080"/>
-          <a:ext cx="1155600" cy="1256760"/>
-        </a:xfrm>
-        <a:prstGeom prst="trapezoid">
-          <a:avLst>
-            <a:gd name="adj" fmla="val 25000"/>
-          </a:avLst>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="dce6f1"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>59</xdr:col>
-      <xdr:colOff>110520</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>61</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="shape325"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="13747680" y="5695920"/>
-          <a:ext cx="461880" cy="334800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="dce6f1"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
       <xdr:col>60</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:colOff>176760</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>60</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:colOff>176760</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>209520</xdr:rowOff>
+      <xdr:rowOff>125640</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="26" name="line326"/>
+        <xdr:cNvPr id="18" name="line315"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="13978440" y="2552760"/>
-          <a:ext cx="360" cy="628920"/>
+          <a:off x="14045040" y="2552760"/>
+          <a:ext cx="360" cy="545040"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3823,26 +3375,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>45</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:col>47</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>60</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:colOff>176760</xdr:colOff>
       <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="27" name="line327"/>
+        <xdr:cNvPr id="19" name="line316"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="10511640" y="2552760"/>
-          <a:ext cx="3467160" cy="360"/>
+          <a:off x="10863720" y="2552760"/>
+          <a:ext cx="3181680" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3859,26 +3411,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>45</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:col>47</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
+      <xdr:rowOff>83520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>45</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:col>47</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>209520</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="28" name="line328"/>
+        <xdr:cNvPr id="20" name="line317"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="10511640" y="2259360"/>
-          <a:ext cx="360" cy="293760"/>
+          <a:off x="10863720" y="2217240"/>
+          <a:ext cx="360" cy="335880"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -3896,140 +3448,26 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
-      <xdr:col>46</xdr:col>
-      <xdr:colOff>176760</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>50</xdr:col>
-      <xdr:colOff>43920</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="shape329"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="10809360" y="1085760"/>
-          <a:ext cx="791640" cy="544320"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="d6cdb4"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>43</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>132480</xdr:colOff>
+      <xdr:row>4</xdr:row>
       <xdr:rowOff>41760</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>48</xdr:col>
-      <xdr:colOff>43920</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="shape330"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9938880" y="1127520"/>
-          <a:ext cx="1199880" cy="1131480"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="d6cdb4"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:round/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr lIns="0" rIns="0" tIns="45000" bIns="45000" anchor="ctr">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="1" lang="en-US" sz="1200" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Arial"/>
-            </a:rPr>
-            <a:t>Dryer Fan</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="en-US" sz="1200" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>50</xdr:col>
-      <xdr:colOff>43920</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>52</xdr:col>
       <xdr:colOff>110160</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>41760</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="31" name="line331"/>
+        <xdr:cNvPr id="21" name="line318"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11601000" y="1357920"/>
-          <a:ext cx="528840" cy="360"/>
+          <a:off x="11458440" y="918000"/>
+          <a:ext cx="671400" cy="360"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4054,18 +3492,18 @@
     <xdr:to>
       <xdr:col>52</xdr:col>
       <xdr:colOff>110160</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>62640</xdr:rowOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>41760</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="32" name="line332"/>
+        <xdr:cNvPr id="22" name="line319"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
           <a:off x="12129480" y="335160"/>
-          <a:ext cx="360" cy="1023120"/>
+          <a:ext cx="360" cy="583200"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4084,25 +3522,25 @@
   <xdr:twoCellAnchor editAs="twoCell">
     <xdr:from>
       <xdr:col>60</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
+      <xdr:colOff>176760</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>41760</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>60</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:colOff>176760</xdr:colOff>
       <xdr:row>30</xdr:row>
       <xdr:rowOff>209520</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="33" name="line333"/>
+        <xdr:cNvPr id="23" name="line320"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13978440" y="6031080"/>
-          <a:ext cx="360" cy="503280"/>
+          <a:off x="14045040" y="6156720"/>
+          <a:ext cx="360" cy="377640"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4133,7 +3571,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="34" name="line334"/>
+        <xdr:cNvPr id="24" name="line321"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -4170,7 +3608,7 @@
     </xdr:to>
     <xdr:cxnSp>
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="35" name="line335"/>
+        <xdr:cNvPr id="25" name="line322"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>

</xml_diff>

<commit_message>
LETEK chicken manure dryer: calculator case run, PFD, and branded budgetary quote
Calculator gains a minimum-drum-diameter input and a case runner.
LETEK case A run through it (XD-96 8x40 selected), Flow PFD exported,
and the budgetary quote PDF built from the repo quote template with
HubSpot export pricing and the PFD appended.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JENvqvx6kQMXayxjNDWASq
</commit_message>
<xml_diff>
--- a/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
+++ b/docs/engineering/dryer-hmb-calculator/MCE_Dryer_HMB_Calculator.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="640">
   <si>
     <t xml:space="preserve">MCE DRYER HEAT &amp; MASS BALANCE CALCULATOR  ·  Rev A  ·  8 Sep 2026</t>
   </si>
@@ -662,6 +662,12 @@
   </si>
   <si>
     <t xml:space="preserve">Model selection margin on airflow and evaporation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum drum diameter (0 = automatic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Force a larger drum than the automatic pick, e.g. 10 for an XD-120</t>
   </si>
   <si>
     <t xml:space="preserve">Burner face heat release</t>
@@ -4005,46 +4011,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="16" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="6" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
       <c r="G4" s="10" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="16" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>2000</v>
@@ -4053,7 +4059,7 @@
         <v>32</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="G6" s="70" t="n">
         <v>480</v>
@@ -4064,7 +4070,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C7" s="25" t="n">
         <v>0.1</v>
@@ -4079,7 +4085,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="C8" s="21" t="n">
         <v>150</v>
@@ -4088,7 +4094,7 @@
         <v>38</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="G8" s="70" t="n">
         <v>750</v>
@@ -4099,7 +4105,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="C9" s="21" t="n">
         <v>8000</v>
@@ -4108,7 +4114,7 @@
         <v>44</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G9" s="70" t="n">
         <v>840</v>
@@ -4119,7 +4125,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C10" s="25" t="n">
         <v>0.02</v>
@@ -4134,7 +4140,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="C11" s="21" t="n">
         <v>932</v>
@@ -4143,7 +4149,7 @@
         <v>38</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="G11" s="70" t="n">
         <v>1100</v>
@@ -4154,16 +4160,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>0.28</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G12" s="70" t="n">
         <v>1300</v>
@@ -4174,7 +4180,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="C13" s="21" t="n">
         <v>12500</v>
@@ -4183,29 +4189,29 @@
         <v>44</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C14" s="21" t="n">
         <v>100</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>0.35</v>
@@ -4216,7 +4222,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="C16" s="21" t="n">
         <v>900</v>
@@ -4227,21 +4233,21 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="C17" s="23" t="n">
         <v>0.05</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="C18" s="23" t="n">
         <v>0.9</v>
@@ -4250,12 +4256,12 @@
         <v>169</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="C19" s="21" t="n">
         <v>1600</v>
@@ -4264,12 +4270,12 @@
         <v>38</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="C20" s="21" t="n">
         <v>700</v>
@@ -4278,12 +4284,12 @@
         <v>38</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C21" s="21" t="n">
         <v>30</v>
@@ -4292,12 +4298,12 @@
         <v>57</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="C22" s="23" t="n">
         <v>0.15</v>
@@ -4308,7 +4314,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="C23" s="27" t="n">
         <v>8</v>
@@ -4319,7 +4325,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="C24" s="27" t="n">
         <v>5</v>
@@ -4328,26 +4334,26 @@
         <v>52</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="8" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="C25" s="21" t="n">
         <v>4000</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
@@ -4355,7 +4361,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="C27" s="29" t="n">
         <f aca="false">IF('Biochar Reactor'!$C$5="Dryer product",HMB!$C$7,'Biochar Reactor'!$C$6)</f>
@@ -4367,7 +4373,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="C28" s="64" t="n">
         <f aca="false">IF('Biochar Reactor'!$C$5="Dryer product",Inputs!$C$15,'Biochar Reactor'!$C$7)</f>
@@ -4377,7 +4383,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="8" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="C29" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$27*(1-'Biochar Reactor'!$C$28)</f>
@@ -4389,7 +4395,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="C30" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$27*'Biochar Reactor'!$C$28</f>
@@ -4401,7 +4407,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="10" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C31" s="59" t="n">
         <f aca="false">'Biochar Reactor'!$C$29*'Biochar Reactor'!$C$12</f>
@@ -4413,19 +4419,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="8" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">'Biochar Reactor'!$C$31/2000</f>
         <v>0.21</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="8" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="C33" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$29-'Biochar Reactor'!$C$31</f>
@@ -4437,7 +4443,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="8" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C34" s="64" t="n">
         <f aca="false">'Biochar Reactor'!$C$31/'Biochar Reactor'!$C$27</f>
@@ -4447,7 +4453,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C35" s="7"/>
       <c r="D35" s="7"/>
@@ -4455,67 +4461,67 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="C36" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$29*'Biochar Reactor'!$C$15*('Biochar Reactor'!$C$11-'Biochar Reactor'!$C$8)</f>
         <v>410550</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="8" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="C37" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$30*(1.01*(212-'Biochar Reactor'!$C$8)+970.4+0.45*('Biochar Reactor'!$C$16-212))</f>
         <v>223770</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="8" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C38" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$29*'Biochar Reactor'!$C$14</f>
         <v>150000</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="C39" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$33*0.45*MAX(0,'Biochar Reactor'!$C$16-'Biochar Reactor'!$C$11)</f>
         <v>0</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="10" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="C40" s="59" t="n">
         <f aca="false">('Biochar Reactor'!$C$36+'Biochar Reactor'!$C$37+'Biochar Reactor'!$C$38+'Biochar Reactor'!$C$39)*(1+'Biochar Reactor'!$C$17)</f>
         <v>823536</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="8" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="C41" s="31" t="n">
         <f aca="false">'Biochar Reactor'!$C$40/1000000</f>
@@ -4527,22 +4533,22 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="C42" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$29*'Biochar Reactor'!$C$9*(1-'Biochar Reactor'!$C$10)-'Biochar Reactor'!$C$31*'Biochar Reactor'!$C$13</f>
         <v>6510000</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="C43" s="31" t="n">
         <f aca="false">'Biochar Reactor'!$C$42/1000000</f>
@@ -4554,19 +4560,19 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="C44" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$42*'Biochar Reactor'!$C$18</f>
         <v>5859000</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="8" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="C45" s="61" t="n">
         <f aca="false">('Biochar Reactor'!$C$19-'Biochar Reactor'!$C$20)/('Biochar Reactor'!$C$19-Inputs!$C$25)</f>
@@ -4576,54 +4582,54 @@
         <v>169</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="8" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C46" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$44*'Biochar Reactor'!$C$45</f>
         <v>3424090.90909091</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="10" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="C47" s="59" t="n">
         <f aca="false">MAX(0,'Biochar Reactor'!$C$40-'Biochar Reactor'!$C$46)</f>
         <v>0</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E47" s="16" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="10" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C48" s="59" t="n">
         <f aca="false">MAX(0,'Biochar Reactor'!$C$44-'Biochar Reactor'!$C$40)</f>
         <v>5035464</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E48" s="16" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="8" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="C49" s="31" t="n">
         <f aca="false">'Biochar Reactor'!$C$48/1000000</f>
@@ -4635,7 +4641,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="8" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C50" s="29" t="str">
         <f aca="false">IF('Biochar Reactor'!$C$47=0,"AUTOTHERMAL: volatiles cover the reactor","NEEDS "&amp;TEXT('Biochar Reactor'!$C$47/1000000,"0.00")&amp;" MMBtu/hr AUXILIARY FUEL")</f>
@@ -4645,7 +4651,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="8" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="C51" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$44/(0.27*('Biochar Reactor'!$C$19-Inputs!$C$25))</f>
@@ -4655,12 +4661,12 @@
         <v>32</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="8" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="C52" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$51/(0.0765*530/(460+'Biochar Reactor'!$C$19))/60</f>
@@ -4672,7 +4678,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="6" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
@@ -4680,31 +4686,31 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="8" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="C54" s="29" t="n">
         <f aca="false">'Biochar Reactor'!$C$27/60/'Biochar Reactor'!$C$23*'Biochar Reactor'!$C$21/'Biochar Reactor'!$C$22</f>
         <v>694.444444444445</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="8" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="C55" s="60" t="n">
         <f aca="false">PI()/4*'Biochar Reactor'!$C$24^2</f>
         <v>19.6349540849362</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="10" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="C56" s="62" t="n">
         <f aca="false">'Biochar Reactor'!$C$54/'Biochar Reactor'!$C$55</f>
@@ -4716,31 +4722,31 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="8" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="C57" s="29" t="n">
         <f aca="false">PI()*'Biochar Reactor'!$C$24*'Biochar Reactor'!$C$56</f>
         <v>555.555555555556</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="10" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C58" s="59" t="n">
         <f aca="false">'Biochar Reactor'!$C$40/'Biochar Reactor'!$C$57</f>
         <v>1482.3648</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="10" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="C59" s="62" t="n">
         <f aca="false">'Biochar Reactor'!$C$40/'Biochar Reactor'!$C$25/(PI()*'Biochar Reactor'!$C$24)</f>
@@ -4752,7 +4758,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="10" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="C60" s="59" t="n">
         <f aca="false">CEILING(MAX('Biochar Reactor'!$C$56,'Biochar Reactor'!$C$59),1)</f>
@@ -4764,7 +4770,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="8" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="C61" s="60" t="n">
         <f aca="false">'Biochar Reactor'!$C$60/'Biochar Reactor'!$C$24</f>
@@ -4772,12 +4778,12 @@
       </c>
       <c r="D61" s="8"/>
       <c r="E61" s="16" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="8" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="C62" s="29" t="str">
         <f aca="false">IF('Biochar Reactor'!$C$58&lt;='Biochar Reactor'!$C$25,"RESIDENCE TIME GOVERNS THE LENGTH","HEAT FLUX GOVERNS: length set by shell area")</f>
@@ -4813,12 +4819,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="6" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -4833,7 +4839,7 @@
         <v>1360.77872830692</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4845,7 +4851,7 @@
         <v>1.36077872830692</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4857,7 +4863,7 @@
         <v>755.988182392733</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4869,12 +4875,12 @@
         <v>604.790545914186</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="C8" s="12" t="str">
         <f aca="false">TEXT(Inputs!$C$14,"0.0%")&amp;" / "&amp;TEXT(Inputs!$C$15,"0.0%")</f>
@@ -4884,7 +4890,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -4892,14 +4898,14 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">HMB!$C$13*2.326</f>
         <v>2614.23792</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4911,43 +4917,43 @@
         <v>4070.5</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="8" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="C12" s="83" t="n">
         <f aca="false">HMB!$C$29*1.05506/1000000</f>
         <v>2.46180666666667</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">HMB!$C$29*0.293071/1000</f>
         <v>683.832333333334</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C14" s="12" t="n">
         <f aca="false">HMB!$C$31/2.20462</f>
         <v>46.4203269890275</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4959,12 +4965,12 @@
         <v>53032.8</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
@@ -4972,31 +4978,31 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="C17" s="12" t="str">
         <f aca="false">TEXT((Inputs!$C$16-32)*5/9,"0")&amp;" / "&amp;TEXT((Inputs!$C$17-32)*5/9,"0")</f>
         <v>16 / 93</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="C18" s="12" t="str">
         <f aca="false">TEXT((Inputs!$C$36-32)*5/9,"0")&amp;" / "&amp;TEXT((Inputs!$C$38-32)*5/9,"0")</f>
         <v>482 / 82</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
@@ -5004,50 +5010,50 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="C20" s="9" t="n">
         <f aca="false">HMB!$C$41/2.20462</f>
         <v>4724.92613995458</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C21" s="9" t="n">
         <f aca="false">HMB!$C$48/2.20462</f>
         <v>5958.16501985915</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C22" s="9" t="n">
         <f aca="false">HMB!$C$53*1.69901</f>
         <v>6607.99972845861</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">HMB!$C$54*1.69901*273.15/294.26</f>
         <v>4959.82423471744</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5060,7 +5066,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="8" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C25" s="12" t="str">
         <f aca="false">Equipment!$C$4</f>
@@ -5070,38 +5076,38 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="C26" s="12" t="str">
         <f aca="false">IF(ISNUMBER(Equipment!$C$5),TEXT(Equipment!$C$5*0.3048,"0.00")&amp;" × "&amp;TEXT(Equipment!$C$6*0.3048,"0.0"),"")</f>
         <v>1.52 × 7.6</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C27" s="11" t="n">
         <f aca="false">Equipment!$C$17*0.293071</f>
         <v>0.8205988</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C28" s="12" t="n">
         <f aca="false">Equipment!$C$27*0.7457</f>
         <v>11.1855</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5113,7 +5119,7 @@
         <v>304.8</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5125,7 +5131,7 @@
         <v>2490.9</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
   </sheetData>
@@ -5154,24 +5160,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="20" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5182,18 +5188,18 @@
         <v>113</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="84" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="C5" s="17" t="n">
         <v>3000</v>
@@ -5210,7 +5216,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="84" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>0.5</v>
@@ -5227,7 +5233,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="84" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>0.1</v>
@@ -5244,7 +5250,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="84" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="C8" s="17" t="n">
         <v>60</v>
@@ -5261,7 +5267,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="84" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="C9" s="17" t="n">
         <v>200</v>
@@ -5278,7 +5284,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="84" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="C10" s="17" t="n">
         <v>600</v>
@@ -5295,7 +5301,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="84" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="C11" s="17" t="n">
         <v>180</v>
@@ -5312,7 +5318,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="84" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C12" s="17" t="n">
         <v>1750</v>
@@ -5349,16 +5355,16 @@
         <v>88</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>
@@ -5859,7 +5865,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:N59"/>
+  <dimension ref="B1:N60"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -6696,75 +6702,78 @@
       <c r="B52" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="C52" s="21" t="n">
-        <v>1200</v>
+      <c r="C52" s="27" t="n">
+        <v>0</v>
       </c>
       <c r="D52" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E52" s="16" t="s">
         <v>210</v>
-      </c>
-      <c r="E52" s="16" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="C53" s="21" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D53" s="8" t="s">
         <v>212</v>
-      </c>
-      <c r="C53" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>169</v>
       </c>
       <c r="E53" s="16" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="6" t="s">
+      <c r="B54" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="7"/>
+      <c r="C54" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E54" s="16" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B55" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="C55" s="17" t="s">
+      <c r="B55" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="D55" s="8"/>
-      <c r="E55" s="16" t="s">
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B56" s="8" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B56" s="6" t="s">
+      <c r="C56" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="7"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="16" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="8" t="s">
-        <v>219</v>
-      </c>
-      <c r="C57" s="21" t="n">
-        <v>24</v>
-      </c>
-      <c r="D57" s="8" t="s">
+      <c r="B57" s="6" t="s">
         <v>220</v>
       </c>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="8" t="s">
         <v>221</v>
       </c>
       <c r="C58" s="21" t="n">
-        <v>312</v>
+        <v>24</v>
       </c>
       <c r="D58" s="8" t="s">
         <v>222</v>
@@ -6774,11 +6783,22 @@
       <c r="B59" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="C59" s="29" t="n">
-        <f aca="false">C57*C58</f>
+      <c r="C59" s="21" t="n">
+        <v>312</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="C60" s="29" t="n">
+        <f aca="false">C58*C59</f>
         <v>7488</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D60" s="8" t="s">
         <v>75</v>
       </c>
     </row>
@@ -6792,7 +6812,7 @@
       <formula1>$G$13:$G$18</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C55" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C56" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6820,7 +6840,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C1" s="32" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="G1" s="33" t="str">
         <f aca="false">Inputs!$C$7</f>
@@ -6917,7 +6937,7 @@
       <c r="P3" s="36"/>
       <c r="Q3" s="36"/>
       <c r="U3" s="37" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="V3" s="37"/>
       <c r="W3" s="37"/>
@@ -6954,7 +6974,7 @@
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="BD4" s="38" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="BE4" s="38"/>
       <c r="BF4" s="38"/>
@@ -7007,7 +7027,7 @@
       <c r="BI5" s="41"/>
       <c r="BJ5" s="41"/>
       <c r="BK5" s="42" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="BL5" s="42"/>
       <c r="BM5" s="42"/>
@@ -7053,7 +7073,7 @@
       <c r="BI6" s="44"/>
       <c r="BJ6" s="44"/>
       <c r="BK6" s="45" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="BL6" s="45"/>
       <c r="BM6" s="45"/>
@@ -7101,7 +7121,7 @@
       <c r="G8" s="48"/>
       <c r="H8" s="48"/>
       <c r="J8" s="40" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="K8" s="40"/>
       <c r="L8" s="40"/>
@@ -7121,7 +7141,7 @@
       <c r="Z8" s="40"/>
       <c r="AA8" s="40"/>
       <c r="BD8" s="38" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="BE8" s="38"/>
       <c r="BF8" s="38"/>
@@ -7146,7 +7166,7 @@
       <c r="BI9" s="41"/>
       <c r="BJ9" s="41"/>
       <c r="BK9" s="42" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="BL9" s="42"/>
       <c r="BM9" s="42"/>
@@ -7154,7 +7174,7 @@
     </row>
     <row r="10" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C10" s="38" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D10" s="38"/>
       <c r="E10" s="38"/>
@@ -7176,7 +7196,7 @@
       <c r="AE10" s="49"/>
       <c r="AF10" s="49"/>
       <c r="AG10" s="50" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="AH10" s="50"/>
       <c r="AI10" s="50"/>
@@ -7201,7 +7221,7 @@
       <c r="BI10" s="44"/>
       <c r="BJ10" s="44"/>
       <c r="BK10" s="45" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="BL10" s="45"/>
       <c r="BM10" s="45"/>
@@ -7219,7 +7239,7 @@
       <c r="H11" s="51"/>
       <c r="I11" s="51"/>
       <c r="J11" s="42" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="K11" s="42"/>
       <c r="L11" s="42"/>
@@ -7237,7 +7257,7 @@
       <c r="H12" s="41"/>
       <c r="I12" s="41"/>
       <c r="J12" s="42" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K12" s="42"/>
       <c r="L12" s="42"/>
@@ -7255,13 +7275,13 @@
       <c r="H13" s="41"/>
       <c r="I13" s="41"/>
       <c r="J13" s="42" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="K13" s="42"/>
       <c r="L13" s="42"/>
       <c r="M13" s="42"/>
       <c r="O13" s="38" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="P13" s="38"/>
       <c r="Q13" s="38"/>
@@ -7272,7 +7292,7 @@
       <c r="V13" s="38"/>
       <c r="W13" s="38"/>
       <c r="AB13" s="38" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="AC13" s="38"/>
       <c r="AD13" s="38"/>
@@ -7296,7 +7316,7 @@
       <c r="H14" s="52"/>
       <c r="I14" s="52"/>
       <c r="J14" s="45" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="K14" s="45"/>
       <c r="L14" s="45"/>
@@ -7310,7 +7330,7 @@
       <c r="R14" s="41"/>
       <c r="S14" s="41"/>
       <c r="T14" s="42" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="U14" s="42"/>
       <c r="V14" s="42"/>
@@ -7325,7 +7345,7 @@
       <c r="AF14" s="41"/>
       <c r="AG14" s="41"/>
       <c r="AH14" s="42" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="AI14" s="42"/>
       <c r="AJ14" s="42"/>
@@ -7341,7 +7361,7 @@
       <c r="R15" s="44"/>
       <c r="S15" s="44"/>
       <c r="T15" s="45" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="U15" s="45"/>
       <c r="V15" s="45"/>
@@ -7356,7 +7376,7 @@
       <c r="AF15" s="44"/>
       <c r="AG15" s="44"/>
       <c r="AH15" s="45" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="AI15" s="45"/>
       <c r="AJ15" s="45"/>
@@ -7372,7 +7392,7 @@
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="X24" s="38" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="Y24" s="38"/>
       <c r="Z24" s="38"/>
@@ -7397,7 +7417,7 @@
       <c r="AC25" s="53"/>
       <c r="AD25" s="53"/>
       <c r="AE25" s="42" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="AF25" s="42"/>
       <c r="AG25" s="42"/>
@@ -7405,7 +7425,7 @@
     </row>
     <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C26" s="38" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D26" s="38"/>
       <c r="E26" s="38"/>
@@ -7428,13 +7448,13 @@
       <c r="AC26" s="41"/>
       <c r="AD26" s="41"/>
       <c r="AE26" s="42" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="AF26" s="42"/>
       <c r="AG26" s="42"/>
       <c r="AH26" s="42"/>
       <c r="AL26" s="34" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="AM26" s="34"/>
       <c r="AN26" s="34"/>
@@ -7459,7 +7479,7 @@
       <c r="H27" s="41"/>
       <c r="I27" s="41"/>
       <c r="J27" s="42" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="K27" s="42"/>
       <c r="L27" s="42"/>
@@ -7475,7 +7495,7 @@
       <c r="AC27" s="41"/>
       <c r="AD27" s="41"/>
       <c r="AE27" s="42" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="AF27" s="42"/>
       <c r="AG27" s="42"/>
@@ -7489,7 +7509,7 @@
       <c r="AO27" s="54"/>
       <c r="AP27" s="54"/>
       <c r="AQ27" s="33" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="AR27" s="33"/>
       <c r="AS27" s="33"/>
@@ -7509,7 +7529,7 @@
       <c r="H28" s="41"/>
       <c r="I28" s="41"/>
       <c r="J28" s="42" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K28" s="42"/>
       <c r="L28" s="42"/>
@@ -7525,7 +7545,7 @@
       <c r="AC28" s="44"/>
       <c r="AD28" s="44"/>
       <c r="AE28" s="45" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="AF28" s="45"/>
       <c r="AG28" s="45"/>
@@ -7543,7 +7563,7 @@
       <c r="H29" s="55"/>
       <c r="I29" s="55"/>
       <c r="J29" s="45" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="K29" s="45"/>
       <c r="L29" s="45"/>
@@ -7571,7 +7591,7 @@
     </row>
     <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="AM30" s="38" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="AN30" s="38"/>
       <c r="AO30" s="38"/>
@@ -7594,7 +7614,7 @@
       <c r="AQ31" s="44"/>
       <c r="AR31" s="44"/>
       <c r="AS31" s="45" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="AT31" s="45"/>
       <c r="AU31" s="45"/>
@@ -7602,7 +7622,7 @@
     </row>
     <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="BD32" s="38" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="BE32" s="38"/>
       <c r="BF32" s="38"/>
@@ -7627,7 +7647,7 @@
       <c r="BI33" s="53"/>
       <c r="BJ33" s="53"/>
       <c r="BK33" s="42" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="BL33" s="42"/>
       <c r="BM33" s="42"/>
@@ -7635,7 +7655,7 @@
     </row>
     <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="AM34" s="38" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AN34" s="38"/>
       <c r="AO34" s="38"/>
@@ -7657,7 +7677,7 @@
       <c r="BI34" s="41"/>
       <c r="BJ34" s="41"/>
       <c r="BK34" s="42" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="BL34" s="42"/>
       <c r="BM34" s="42"/>
@@ -7674,7 +7694,7 @@
       <c r="AQ35" s="44"/>
       <c r="AR35" s="44"/>
       <c r="AS35" s="45" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="AT35" s="45"/>
       <c r="AU35" s="45"/>
@@ -7690,7 +7710,7 @@
       <c r="BI35" s="41"/>
       <c r="BJ35" s="41"/>
       <c r="BK35" s="42" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="BL35" s="42"/>
       <c r="BM35" s="42"/>
@@ -7708,7 +7728,7 @@
       <c r="BI36" s="41"/>
       <c r="BJ36" s="41"/>
       <c r="BK36" s="42" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="BL36" s="42"/>
       <c r="BM36" s="42"/>
@@ -7726,7 +7746,7 @@
       <c r="BI37" s="44"/>
       <c r="BJ37" s="44"/>
       <c r="BK37" s="45" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="BL37" s="45"/>
       <c r="BM37" s="45"/>
@@ -7775,7 +7795,7 @@
       <c r="AD47" s="33"/>
       <c r="AE47" s="33"/>
       <c r="AF47" s="57" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AG47" s="57"/>
       <c r="AH47" s="57"/>
@@ -7797,7 +7817,7 @@
       <c r="AX47" s="57"/>
       <c r="AY47" s="57"/>
       <c r="BG47" s="58" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="BH47" s="58"/>
       <c r="BI47" s="58"/>
@@ -7927,12 +7947,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -7952,7 +7972,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C5" s="29" t="n">
         <f aca="false">Inputs!$C$13*(1-Inputs!$C$14)</f>
@@ -7964,7 +7984,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C6" s="29" t="n">
         <f aca="false">Inputs!$C$13*Inputs!$C$14</f>
@@ -7988,7 +8008,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C8" s="29" t="n">
         <f aca="false">HMB!$C$7-HMB!$C$5</f>
@@ -8010,7 +8030,7 @@
         <v>32</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8022,24 +8042,24 @@
         <v>159.776313161574</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">HMB!$C$7/2000</f>
         <v>0.833333333333333</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -8047,7 +8067,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C13" s="60" t="n">
         <f aca="false">1.01*(212-Inputs!$C$16)+970.4</f>
@@ -8057,12 +8077,12 @@
         <v>44</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">Inputs!$C$29</f>
@@ -8074,22 +8094,22 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="10" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C15" s="59" t="n">
         <f aca="false">HMB!$C$9*HMB!$C$14</f>
         <v>2333333.33333333</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C16" s="31" t="n">
         <f aca="false">HMB!$C$15/1000000</f>
@@ -8101,7 +8121,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
@@ -8109,82 +8129,82 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C18" s="29" t="n">
         <f aca="false">HMB!$C$5*Inputs!$C$18*(Inputs!$C$17-Inputs!$C$16)</f>
         <v>73500</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C19" s="29" t="n">
         <f aca="false">HMB!$C$8*1*(Inputs!$C$17-Inputs!$C$16)</f>
         <v>23333.3333333333</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C20" s="29" t="n">
         <f aca="false">HMB!$C$9*1.01*(212-Inputs!$C$16)</f>
         <v>204693.333333333</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C21" s="29" t="n">
         <f aca="false">HMB!$C$9*970.4</f>
         <v>1293866.66666667</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C22" s="29" t="n">
         <f aca="false">HMB!$C$9*0.45*(Inputs!$C$38-212)</f>
         <v>-19200</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="10" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C23" s="59" t="n">
         <f aca="false">SUM($C$18:$C$22)</f>
         <v>1576193.33333333</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C24" s="61" t="n">
         <f aca="false">Inputs!$C$39*(Inputs!$C$36-Inputs!$C$38)/(Inputs!$C$36-Inputs!$C$25)</f>
@@ -8194,27 +8214,27 @@
         <v>169</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="10" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C25" s="59" t="n">
         <f aca="false">HMB!$C$23/(HMB!$C$24-Inputs!$C$40)</f>
         <v>2125886.96210662</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C26" s="31" t="n">
         <f aca="false">HMB!$C$25/1000000</f>
@@ -8238,7 +8258,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C28" s="29" t="str">
         <f aca="false">IF(ABS(HMB!$C$27/HMB!$C$14-1)&lt;=0.15,"WITHIN 15% OF MCE FACTOR",IF(HMB!$C$27&gt;HMB!$C$14,"RIGOROUS IS HIGHER: raise inlet temp or accept higher fuel","RIGOROUS IS LOWER: MCE factor is conservative here"))</f>
@@ -8246,27 +8266,27 @@
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="16" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="10" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C29" s="59" t="n">
         <f aca="false">MAX(HMB!$C$15,HMB!$C$25)</f>
         <v>2333333.33333333</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
@@ -8274,7 +8294,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="10" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C31" s="62" t="n">
         <f aca="false">HMB!$C$29/Inputs!$C$31</f>
@@ -8286,34 +8306,34 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="8" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C32" s="29" t="n">
-        <f aca="false">IF(Inputs!$C$55="Yes",MAX(0,MIN(HMB!$C$29,'Biochar Reactor'!$C$48)),0)</f>
+        <f aca="false">IF(Inputs!$C$56="Yes",MAX(0,MIN(HMB!$C$29,'Biochar Reactor'!$C$48)),0)</f>
         <v>0</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="10" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C33" s="59" t="n">
         <f aca="false">HMB!$C$29-HMB!$C$32</f>
         <v>2333333.33333333</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="10" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C34" s="62" t="n">
         <f aca="false">HMB!$C$33/Inputs!$C$31</f>
@@ -8325,22 +8345,22 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="8" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C35" s="60" t="n">
         <f aca="false">HMB!$C$31/INDEX(Inputs!$I$13:$I$18,MATCH(Inputs!$C$30,Inputs!$G$13:$G$18,0))/60</f>
         <v>38.7648413964204</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C36" s="29" t="n">
         <f aca="false">HMB!$C$31*Inputs!$C$33*(1+Inputs!$C$32)</f>
@@ -8352,7 +8372,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="8" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C37" s="29" t="n">
         <f aca="false">HMB!$C$31+HMB!$C$36</f>
@@ -8364,7 +8384,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="8" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C38" s="29" t="n">
         <f aca="false">HMB!$C$31*Inputs!$C$34+HMB!$C$36*Inputs!$C$26</f>
@@ -8376,7 +8396,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C39" s="29" t="n">
         <f aca="false">Inputs!$C$25+HMB!$C$29*Inputs!$C$39/(0.27*HMB!$C$37)</f>
@@ -8386,12 +8406,12 @@
         <v>38</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="6" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
@@ -8399,7 +8419,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="10" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C41" s="59" t="n">
         <f aca="false">HMB!$C$29*Inputs!$C$39/(0.24*(Inputs!$C$36-Inputs!$C$25))</f>
@@ -8409,12 +8429,12 @@
         <v>32</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C42" s="29" t="n">
         <f aca="false">HMB!$C$41-HMB!$C$37</f>
@@ -8424,12 +8444,12 @@
         <v>32</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C43" s="29" t="str">
         <f aca="false">IF(Inputs!$C$36&lt;=Inputs!$C$37,"OK","INLET ABOVE MCE MAXIMUM - lower it")</f>
@@ -8439,7 +8459,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C44" s="29" t="str">
         <f aca="false">IF(HMB!$C$42&lt;0,"INLET TEMP TOO HIGH FOR THIS FUEL / EXCESS AIR","OK")</f>
@@ -8449,7 +8469,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="8" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C45" s="29" t="n">
         <f aca="false">HMB!$C$41*Inputs!$C$41</f>
@@ -8461,7 +8481,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="8" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C46" s="29" t="n">
         <f aca="false">HMB!$C$41+HMB!$C$45</f>
@@ -8473,7 +8493,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="8" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C47" s="29" t="n">
         <f aca="false">HMB!$C$38+(HMB!$C$42+HMB!$C$45)*Inputs!$C$26+HMB!$C$9</f>
@@ -8485,7 +8505,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="10" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C48" s="59" t="n">
         <f aca="false">HMB!$C$46+HMB!$C$47</f>
@@ -8497,19 +8517,19 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="8" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C49" s="61" t="n">
         <f aca="false">HMB!$C$47/HMB!$C$46</f>
         <v>0.146370015948963</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C50" s="63" t="n">
         <f aca="false">(1-0.0000068754*Inputs!$C$24)^5.2559</f>
@@ -8517,12 +8537,12 @@
       </c>
       <c r="D50" s="8"/>
       <c r="E50" s="16" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="8" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C51" s="63" t="n">
         <f aca="false">0.0765*530/(460+Inputs!$C$38)*HMB!$C$50</f>
@@ -8534,7 +8554,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="8" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C52" s="63" t="n">
         <f aca="false">0.0476*530/(460+Inputs!$C$38)*HMB!$C$50</f>
@@ -8546,7 +8566,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B53" s="10" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C53" s="59" t="n">
         <f aca="false">HMB!$C$46/HMB!$C$51/60+HMB!$C$47/HMB!$C$52/60</f>
@@ -8556,48 +8576,48 @@
         <v>66</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="8" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C54" s="29" t="n">
         <f aca="false">HMB!$C$46/0.075/60+HMB!$C$47/0.0467/60</f>
         <v>3144.85319592104</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B55" s="8" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C55" s="29" t="n">
         <f aca="false">HMB!$C$41/0.075/60</f>
         <v>2314.81481481482</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B56" s="8" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C56" s="29" t="n">
         <f aca="false">HMB!$C$42/0.075/60</f>
         <v>1827.85087719298</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="8" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C57" s="29" t="n">
         <f aca="false">HMB!$C$36/(0.0765*530/(460+Inputs!$C$25)*HMB!$C$50)/60</f>
@@ -8609,7 +8629,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B58" s="8" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C58" s="60" t="n">
         <f aca="false">IF(OR(Inputs!$C$30="Dry Wood",Inputs!$C$30="Biomass (wet, 8,500)"),HMB!$C$34,0)</f>
@@ -8619,12 +8639,12 @@
         <v>32</v>
       </c>
       <c r="E58" s="16" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="8" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C59" s="29" t="n">
         <f aca="false">HMB!$C$7-HMB!$C$58</f>
@@ -8636,7 +8656,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="8" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C60" s="29" t="n">
         <f aca="false">(HMB!$C$41/(0.0765*530/(460+Inputs!$C$36)*HMB!$C$50)+HMB!$C$38/(0.0476*530/(460+Inputs!$C$36)*HMB!$C$50))/60</f>
@@ -8646,12 +8666,12 @@
         <v>66</v>
       </c>
       <c r="E60" s="16" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="8" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C61" s="60" t="n">
         <f aca="false">HMB!$C$46/HMB!$C$7</f>
@@ -8663,7 +8683,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B62" s="8" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C62" s="29" t="str">
         <f aca="false">IF(HMB!$C$61&gt;=Inputs!$C$49,"CONVEYING CAN OCCUR","CONVEYING CANNOT OCCUR: add recycle or raise airflow")</f>
@@ -8673,7 +8693,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="6" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C63" s="7"/>
       <c r="D63" s="7"/>
@@ -8681,85 +8701,85 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="8" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C64" s="29" t="n">
         <f aca="false">HMB!$C$29</f>
         <v>2333333.33333333</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="8" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C65" s="29" t="n">
         <f aca="false">HMB!$C$29*(1-Inputs!$C$39)</f>
         <v>233333.333333333</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="8" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C66" s="29" t="n">
         <f aca="false">HMB!$C$23*HMB!$C$29/HMB!$C$25</f>
         <v>1730000</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E66" s="16" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="8" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C67" s="29" t="n">
         <f aca="false">HMB!$C$29*Inputs!$C$40</f>
         <v>70000</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B68" s="8" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C68" s="29" t="n">
         <f aca="false">HMB!$C$41*0.24*(Inputs!$C$38-Inputs!$C$25)</f>
         <v>300000</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B69" s="10" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C69" s="59" t="n">
         <f aca="false">HMB!$C$64-HMB!$C$65-HMB!$C$66-HMB!$C$67-HMB!$C$68</f>
         <v>0</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E69" s="16" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B70" s="8" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C70" s="64" t="n">
         <f aca="false">HMB!$C$69/HMB!$C$64</f>
@@ -8769,7 +8789,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B71" s="6" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C71" s="7"/>
       <c r="D71" s="7"/>
@@ -8777,7 +8797,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B72" s="8" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C72" s="9" t="str">
         <f aca="false">Equipment!$C$4</f>
@@ -8787,19 +8807,19 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B73" s="8" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C73" s="9" t="n">
         <f aca="false">Equipment!$C$7</f>
         <v>490.873852123405</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B74" s="10" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C74" s="65" t="n">
         <f aca="false">IF(HMB!$C$73&gt;0,HMB!$C$9/HMB!$C$73,"n/a")</f>
@@ -8809,24 +8829,24 @@
         <v>59</v>
       </c>
       <c r="E74" s="16" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B75" s="8" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C75" s="60" t="n">
         <f aca="false">Inputs!$C$13/60*Inputs!$C$21/Inputs!$C$20</f>
         <v>62.5</v>
       </c>
       <c r="D75" s="8" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B76" s="8" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C76" s="64" t="n">
         <f aca="false">IF(HMB!$C$73&gt;0,HMB!$C$75/HMB!$C$73,"n/a")</f>
@@ -8836,12 +8856,12 @@
         <v>169</v>
       </c>
       <c r="E76" s="16" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B77" s="8" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C77" s="60" t="n">
         <f aca="false">IF(HMB!$C$73&gt;0,HMB!$C$73*Inputs!$C$22/(Inputs!$C$13/60/Inputs!$C$20),"n/a")</f>
@@ -8853,19 +8873,19 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="8" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C78" s="29" t="n">
         <f aca="false">HMB!$C$75/Inputs!$C$22</f>
         <v>625</v>
       </c>
       <c r="D78" s="8" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B79" s="10" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C79" s="62" t="n">
         <f aca="false">IF(ISNUMBER(Equipment!$C$5),HMB!$C$78/(PI()/4*Equipment!$C$5^2),"n/a")</f>
@@ -8875,12 +8895,12 @@
         <v>52</v>
       </c>
       <c r="E79" s="16" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B80" s="10" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C80" s="59" t="n">
         <f aca="false">IF(ISNUMBER(Equipment!$C$6),MAX(Equipment!$C$6,CEILING(HMB!$C$79,1)),"n/a")</f>
@@ -8935,27 +8955,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="8" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="K2" s="66" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="L2" s="67" t="n">
         <v>6</v>
       </c>
       <c r="M2" s="66" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="N2" s="67" t="n">
         <v>8</v>
       </c>
       <c r="O2" s="66" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="P2" s="67" t="n">
         <v>8</v>
@@ -8963,57 +8983,57 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="16" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="20" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C5" s="20" t="s">
         <v>50</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="K5" s="20" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="L5" s="20" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="M5" s="20" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="N5" s="20" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="O5" s="20" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="P5" s="20" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="Q5" s="20" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9021,7 +9041,7 @@
         <v>95</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>3</v>
@@ -9055,7 +9075,7 @@
         <v>508.938009881546</v>
       </c>
       <c r="M6" s="69" t="n">
-        <f aca="false">IF(AND(B6=Inputs!$C$28,H6&lt;&gt;"",L6&lt;&gt;"",H6&gt;=HMB!$C$53*(1+Inputs!$C$51),L6&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B6=Inputs!$C$28,H6&lt;&gt;"",L6&lt;&gt;"",D6&gt;=Inputs!$C$52,H6&gt;=HMB!$C$53*(1+Inputs!$C$51),L6&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N6" s="68" t="n">
@@ -9065,7 +9085,7 @@
       <c r="O6" s="70"/>
       <c r="P6" s="71"/>
       <c r="Q6" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9073,7 +9093,7 @@
         <v>95</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D7" s="17" t="n">
         <v>3</v>
@@ -9107,7 +9127,7 @@
         <v>848.230016469244</v>
       </c>
       <c r="M7" s="69" t="n">
-        <f aca="false">IF(AND(B7=Inputs!$C$28,H7&lt;&gt;"",L7&lt;&gt;"",H7&gt;=HMB!$C$53*(1+Inputs!$C$51),L7&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B7=Inputs!$C$28,H7&lt;&gt;"",L7&lt;&gt;"",D7&gt;=Inputs!$C$52,H7&gt;=HMB!$C$53*(1+Inputs!$C$51),L7&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N7" s="68" t="n">
@@ -9117,7 +9137,7 @@
       <c r="O7" s="70"/>
       <c r="P7" s="71"/>
       <c r="Q7" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9125,7 +9145,7 @@
         <v>95</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="D8" s="17" t="n">
         <v>4</v>
@@ -9159,7 +9179,7 @@
         <v>1507.9644737231</v>
       </c>
       <c r="M8" s="69" t="n">
-        <f aca="false">IF(AND(B8=Inputs!$C$28,H8&lt;&gt;"",L8&lt;&gt;"",H8&gt;=HMB!$C$53*(1+Inputs!$C$51),L8&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B8=Inputs!$C$28,H8&lt;&gt;"",L8&lt;&gt;"",D8&gt;=Inputs!$C$52,H8&gt;=HMB!$C$53*(1+Inputs!$C$51),L8&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N8" s="68" t="n">
@@ -9169,7 +9189,7 @@
       <c r="O8" s="70"/>
       <c r="P8" s="71"/>
       <c r="Q8" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9177,7 +9197,7 @@
         <v>95</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D9" s="17" t="n">
         <v>5</v>
@@ -9211,7 +9231,7 @@
         <v>2945.24311274043</v>
       </c>
       <c r="M9" s="69" t="n">
-        <f aca="false">IF(AND(B9=Inputs!$C$28,H9&lt;&gt;"",L9&lt;&gt;"",H9&gt;=HMB!$C$53*(1+Inputs!$C$51),L9&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B9=Inputs!$C$28,H9&lt;&gt;"",L9&lt;&gt;"",D9&gt;=Inputs!$C$52,H9&gt;=HMB!$C$53*(1+Inputs!$C$51),L9&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>9</v>
       </c>
       <c r="N9" s="68" t="n">
@@ -9221,7 +9241,7 @@
       <c r="O9" s="70"/>
       <c r="P9" s="71"/>
       <c r="Q9" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9229,7 +9249,7 @@
         <v>95</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D10" s="17" t="n">
         <v>6</v>
@@ -9263,7 +9283,7 @@
         <v>5089.38009881546</v>
       </c>
       <c r="M10" s="69" t="n">
-        <f aca="false">IF(AND(B10=Inputs!$C$28,H10&lt;&gt;"",L10&lt;&gt;"",H10&gt;=HMB!$C$53*(1+Inputs!$C$51),L10&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B10=Inputs!$C$28,H10&lt;&gt;"",L10&lt;&gt;"",D10&gt;=Inputs!$C$52,H10&gt;=HMB!$C$53*(1+Inputs!$C$51),L10&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>10</v>
       </c>
       <c r="N10" s="68" t="n">
@@ -9273,7 +9293,7 @@
       <c r="O10" s="70"/>
       <c r="P10" s="71"/>
       <c r="Q10" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9281,7 +9301,7 @@
         <v>95</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D11" s="17" t="n">
         <v>7</v>
@@ -9315,7 +9335,7 @@
         <v>8081.74710135974</v>
       </c>
       <c r="M11" s="69" t="n">
-        <f aca="false">IF(AND(B11=Inputs!$C$28,H11&lt;&gt;"",L11&lt;&gt;"",H11&gt;=HMB!$C$53*(1+Inputs!$C$51),L11&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B11=Inputs!$C$28,H11&lt;&gt;"",L11&lt;&gt;"",D11&gt;=Inputs!$C$52,H11&gt;=HMB!$C$53*(1+Inputs!$C$51),L11&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>11</v>
       </c>
       <c r="N11" s="68" t="n">
@@ -9325,7 +9345,7 @@
       <c r="O11" s="70"/>
       <c r="P11" s="71"/>
       <c r="Q11" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9333,7 +9353,7 @@
         <v>95</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D12" s="17" t="n">
         <v>8</v>
@@ -9367,7 +9387,7 @@
         <v>12063.7157897848</v>
       </c>
       <c r="M12" s="69" t="n">
-        <f aca="false">IF(AND(B12=Inputs!$C$28,H12&lt;&gt;"",L12&lt;&gt;"",H12&gt;=HMB!$C$53*(1+Inputs!$C$51),L12&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B12=Inputs!$C$28,H12&lt;&gt;"",L12&lt;&gt;"",D12&gt;=Inputs!$C$52,H12&gt;=HMB!$C$53*(1+Inputs!$C$51),L12&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>12</v>
       </c>
       <c r="N12" s="68" t="n">
@@ -9377,7 +9397,7 @@
       <c r="O12" s="70"/>
       <c r="P12" s="71"/>
       <c r="Q12" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9385,7 +9405,7 @@
         <v>95</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D13" s="17" t="n">
         <v>10</v>
@@ -9419,7 +9439,7 @@
         <v>23561.9449019235</v>
       </c>
       <c r="M13" s="69" t="n">
-        <f aca="false">IF(AND(B13=Inputs!$C$28,H13&lt;&gt;"",L13&lt;&gt;"",H13&gt;=HMB!$C$53*(1+Inputs!$C$51),L13&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B13=Inputs!$C$28,H13&lt;&gt;"",L13&lt;&gt;"",D13&gt;=Inputs!$C$52,H13&gt;=HMB!$C$53*(1+Inputs!$C$51),L13&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>13</v>
       </c>
       <c r="N13" s="68" t="n">
@@ -9429,7 +9449,7 @@
       <c r="O13" s="70"/>
       <c r="P13" s="71"/>
       <c r="Q13" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9437,7 +9457,7 @@
         <v>95</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D14" s="17" t="n">
         <v>12</v>
@@ -9471,7 +9491,7 @@
         <v>40715.0407905237</v>
       </c>
       <c r="M14" s="69" t="n">
-        <f aca="false">IF(AND(B14=Inputs!$C$28,H14&lt;&gt;"",L14&lt;&gt;"",H14&gt;=HMB!$C$53*(1+Inputs!$C$51),L14&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B14=Inputs!$C$28,H14&lt;&gt;"",L14&lt;&gt;"",D14&gt;=Inputs!$C$52,H14&gt;=HMB!$C$53*(1+Inputs!$C$51),L14&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>14</v>
       </c>
       <c r="N14" s="68" t="n">
@@ -9481,7 +9501,7 @@
       <c r="O14" s="70"/>
       <c r="P14" s="71"/>
       <c r="Q14" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9489,7 +9509,7 @@
         <v>95</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="D15" s="17" t="n">
         <v>13</v>
@@ -9523,7 +9543,7 @@
         <v>47783.6242611008</v>
       </c>
       <c r="M15" s="69" t="n">
-        <f aca="false">IF(AND(B15=Inputs!$C$28,H15&lt;&gt;"",L15&lt;&gt;"",H15&gt;=HMB!$C$53*(1+Inputs!$C$51),L15&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B15=Inputs!$C$28,H15&lt;&gt;"",L15&lt;&gt;"",D15&gt;=Inputs!$C$52,H15&gt;=HMB!$C$53*(1+Inputs!$C$51),L15&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>15</v>
       </c>
       <c r="N15" s="68" t="n">
@@ -9533,7 +9553,7 @@
       <c r="O15" s="70"/>
       <c r="P15" s="71"/>
       <c r="Q15" s="16" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9541,7 +9561,7 @@
         <v>95</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D16" s="72"/>
       <c r="E16" s="72"/>
@@ -9571,7 +9591,7 @@
         <v/>
       </c>
       <c r="M16" s="69" t="n">
-        <f aca="false">IF(AND(B16=Inputs!$C$28,H16&lt;&gt;"",L16&lt;&gt;"",H16&gt;=HMB!$C$53*(1+Inputs!$C$51),L16&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B16=Inputs!$C$28,H16&lt;&gt;"",L16&lt;&gt;"",D16&gt;=Inputs!$C$52,H16&gt;=HMB!$C$53*(1+Inputs!$C$51),L16&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N16" s="68" t="str">
@@ -9581,7 +9601,7 @@
       <c r="O16" s="70"/>
       <c r="P16" s="71"/>
       <c r="Q16" s="16" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9589,7 +9609,7 @@
         <v>99</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D17" s="17" t="n">
         <v>3</v>
@@ -9606,7 +9626,7 @@
         <v>84.8230016469244</v>
       </c>
       <c r="H17" s="73" t="n">
-        <f aca="false">IF(F17="","",F17*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F17="","",F17*Inputs!$C$44*Inputs!$C$54)</f>
         <v>2474.00421470196</v>
       </c>
       <c r="I17" s="27"/>
@@ -9623,7 +9643,7 @@
         <v>678.584013175395</v>
       </c>
       <c r="M17" s="69" t="n">
-        <f aca="false">IF(AND(B17=Inputs!$C$28,H17&lt;&gt;"",L17&lt;&gt;"",H17&gt;=HMB!$C$53*(1+Inputs!$C$51),L17&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B17=Inputs!$C$28,H17&lt;&gt;"",L17&lt;&gt;"",D17&gt;=Inputs!$C$52,H17&gt;=HMB!$C$53*(1+Inputs!$C$51),L17&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N17" s="68" t="n">
@@ -9633,7 +9653,7 @@
       <c r="O17" s="70"/>
       <c r="P17" s="71"/>
       <c r="Q17" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9641,7 +9661,7 @@
         <v>99</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D18" s="17" t="n">
         <v>3</v>
@@ -9658,7 +9678,7 @@
         <v>141.371669411541</v>
       </c>
       <c r="H18" s="73" t="n">
-        <f aca="false">IF(F18="","",F18*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F18="","",F18*Inputs!$C$44*Inputs!$C$54)</f>
         <v>2474.00421470196</v>
       </c>
       <c r="I18" s="27"/>
@@ -9675,7 +9695,7 @@
         <v>1130.97335529233</v>
       </c>
       <c r="M18" s="69" t="n">
-        <f aca="false">IF(AND(B18=Inputs!$C$28,H18&lt;&gt;"",L18&lt;&gt;"",H18&gt;=HMB!$C$53*(1+Inputs!$C$51),L18&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B18=Inputs!$C$28,H18&lt;&gt;"",L18&lt;&gt;"",D18&gt;=Inputs!$C$52,H18&gt;=HMB!$C$53*(1+Inputs!$C$51),L18&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N18" s="68" t="n">
@@ -9685,7 +9705,7 @@
       <c r="O18" s="70"/>
       <c r="P18" s="71"/>
       <c r="Q18" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9693,7 +9713,7 @@
         <v>99</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="D19" s="17" t="n">
         <v>4</v>
@@ -9710,7 +9730,7 @@
         <v>251.327412287183</v>
       </c>
       <c r="H19" s="73" t="n">
-        <f aca="false">IF(F19="","",F19*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F19="","",F19*Inputs!$C$44*Inputs!$C$54)</f>
         <v>4398.22971502571</v>
       </c>
       <c r="I19" s="27"/>
@@ -9727,7 +9747,7 @@
         <v>2010.61929829747</v>
       </c>
       <c r="M19" s="69" t="n">
-        <f aca="false">IF(AND(B19=Inputs!$C$28,H19&lt;&gt;"",L19&lt;&gt;"",H19&gt;=HMB!$C$53*(1+Inputs!$C$51),L19&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B19=Inputs!$C$28,H19&lt;&gt;"",L19&lt;&gt;"",D19&gt;=Inputs!$C$52,H19&gt;=HMB!$C$53*(1+Inputs!$C$51),L19&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N19" s="68" t="n">
@@ -9737,7 +9757,7 @@
       <c r="O19" s="70"/>
       <c r="P19" s="71"/>
       <c r="Q19" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9745,7 +9765,7 @@
         <v>99</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D20" s="17" t="n">
         <v>5</v>
@@ -9762,7 +9782,7 @@
         <v>490.873852123405</v>
       </c>
       <c r="H20" s="73" t="n">
-        <f aca="false">IF(F20="","",F20*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F20="","",F20*Inputs!$C$44*Inputs!$C$54)</f>
         <v>6872.23392972767</v>
       </c>
       <c r="I20" s="27"/>
@@ -9779,7 +9799,7 @@
         <v>3926.99081698724</v>
       </c>
       <c r="M20" s="69" t="n">
-        <f aca="false">IF(AND(B20=Inputs!$C$28,H20&lt;&gt;"",L20&lt;&gt;"",H20&gt;=HMB!$C$53*(1+Inputs!$C$51),L20&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B20=Inputs!$C$28,H20&lt;&gt;"",L20&lt;&gt;"",D20&gt;=Inputs!$C$52,H20&gt;=HMB!$C$53*(1+Inputs!$C$51),L20&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N20" s="68" t="n">
@@ -9789,7 +9809,7 @@
       <c r="O20" s="70"/>
       <c r="P20" s="71"/>
       <c r="Q20" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9797,7 +9817,7 @@
         <v>99</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="D21" s="17" t="n">
         <v>6</v>
@@ -9814,7 +9834,7 @@
         <v>848.230016469244</v>
       </c>
       <c r="H21" s="73" t="n">
-        <f aca="false">IF(F21="","",F21*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F21="","",F21*Inputs!$C$44*Inputs!$C$54)</f>
         <v>9896.01685880785</v>
       </c>
       <c r="I21" s="27"/>
@@ -9831,7 +9851,7 @@
         <v>6785.84013175395</v>
       </c>
       <c r="M21" s="69" t="n">
-        <f aca="false">IF(AND(B21=Inputs!$C$28,H21&lt;&gt;"",L21&lt;&gt;"",H21&gt;=HMB!$C$53*(1+Inputs!$C$51),L21&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B21=Inputs!$C$28,H21&lt;&gt;"",L21&lt;&gt;"",D21&gt;=Inputs!$C$52,H21&gt;=HMB!$C$53*(1+Inputs!$C$51),L21&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N21" s="68" t="n">
@@ -9841,7 +9861,7 @@
       <c r="O21" s="70"/>
       <c r="P21" s="71"/>
       <c r="Q21" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9849,7 +9869,7 @@
         <v>99</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D22" s="17" t="n">
         <v>7</v>
@@ -9866,7 +9886,7 @@
         <v>1346.95785022662</v>
       </c>
       <c r="H22" s="73" t="n">
-        <f aca="false">IF(F22="","",F22*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F22="","",F22*Inputs!$C$44*Inputs!$C$54)</f>
         <v>13469.5785022662</v>
       </c>
       <c r="I22" s="27"/>
@@ -9883,7 +9903,7 @@
         <v>10775.662801813</v>
       </c>
       <c r="M22" s="69" t="n">
-        <f aca="false">IF(AND(B22=Inputs!$C$28,H22&lt;&gt;"",L22&lt;&gt;"",H22&gt;=HMB!$C$53*(1+Inputs!$C$51),L22&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B22=Inputs!$C$28,H22&lt;&gt;"",L22&lt;&gt;"",D22&gt;=Inputs!$C$52,H22&gt;=HMB!$C$53*(1+Inputs!$C$51),L22&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N22" s="68" t="n">
@@ -9893,7 +9913,7 @@
       <c r="O22" s="70"/>
       <c r="P22" s="71"/>
       <c r="Q22" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9901,7 +9921,7 @@
         <v>99</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D23" s="17" t="n">
         <v>8</v>
@@ -9918,7 +9938,7 @@
         <v>2010.61929829747</v>
       </c>
       <c r="H23" s="73" t="n">
-        <f aca="false">IF(F23="","",F23*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F23="","",F23*Inputs!$C$44*Inputs!$C$54)</f>
         <v>17592.9188601028</v>
       </c>
       <c r="I23" s="27"/>
@@ -9935,7 +9955,7 @@
         <v>16084.9543863797</v>
       </c>
       <c r="M23" s="69" t="n">
-        <f aca="false">IF(AND(B23=Inputs!$C$28,H23&lt;&gt;"",L23&lt;&gt;"",H23&gt;=HMB!$C$53*(1+Inputs!$C$51),L23&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B23=Inputs!$C$28,H23&lt;&gt;"",L23&lt;&gt;"",D23&gt;=Inputs!$C$52,H23&gt;=HMB!$C$53*(1+Inputs!$C$51),L23&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N23" s="68" t="n">
@@ -9945,7 +9965,7 @@
       <c r="O23" s="70"/>
       <c r="P23" s="71"/>
       <c r="Q23" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9953,7 +9973,7 @@
         <v>99</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D24" s="17" t="n">
         <v>10</v>
@@ -9970,7 +9990,7 @@
         <v>3926.99081698724</v>
       </c>
       <c r="H24" s="73" t="n">
-        <f aca="false">IF(F24="","",F24*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F24="","",F24*Inputs!$C$44*Inputs!$C$54)</f>
         <v>27488.9357189107</v>
       </c>
       <c r="I24" s="27"/>
@@ -9987,7 +10007,7 @@
         <v>31415.9265358979</v>
       </c>
       <c r="M24" s="69" t="n">
-        <f aca="false">IF(AND(B24=Inputs!$C$28,H24&lt;&gt;"",L24&lt;&gt;"",H24&gt;=HMB!$C$53*(1+Inputs!$C$51),L24&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B24=Inputs!$C$28,H24&lt;&gt;"",L24&lt;&gt;"",D24&gt;=Inputs!$C$52,H24&gt;=HMB!$C$53*(1+Inputs!$C$51),L24&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N24" s="68" t="n">
@@ -9997,7 +10017,7 @@
       <c r="O24" s="70"/>
       <c r="P24" s="71"/>
       <c r="Q24" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10005,7 +10025,7 @@
         <v>99</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="D25" s="17" t="n">
         <v>12</v>
@@ -10022,7 +10042,7 @@
         <v>6785.84013175395</v>
       </c>
       <c r="H25" s="73" t="n">
-        <f aca="false">IF(F25="","",F25*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F25="","",F25*Inputs!$C$44*Inputs!$C$54)</f>
         <v>39584.0674352314</v>
       </c>
       <c r="I25" s="27"/>
@@ -10039,7 +10059,7 @@
         <v>54286.7210540316</v>
       </c>
       <c r="M25" s="69" t="n">
-        <f aca="false">IF(AND(B25=Inputs!$C$28,H25&lt;&gt;"",L25&lt;&gt;"",H25&gt;=HMB!$C$53*(1+Inputs!$C$51),L25&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B25=Inputs!$C$28,H25&lt;&gt;"",L25&lt;&gt;"",D25&gt;=Inputs!$C$52,H25&gt;=HMB!$C$53*(1+Inputs!$C$51),L25&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N25" s="68" t="n">
@@ -10049,7 +10069,7 @@
       <c r="O25" s="70"/>
       <c r="P25" s="71"/>
       <c r="Q25" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10057,7 +10077,7 @@
         <v>99</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D26" s="17" t="n">
         <v>13</v>
@@ -10074,7 +10094,7 @@
         <v>7963.93737685013</v>
       </c>
       <c r="H26" s="73" t="n">
-        <f aca="false">IF(F26="","",F26*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F26="","",F26*Inputs!$C$44*Inputs!$C$54)</f>
         <v>46456.3013649591</v>
       </c>
       <c r="I26" s="27"/>
@@ -10091,7 +10111,7 @@
         <v>63711.499014801</v>
       </c>
       <c r="M26" s="69" t="n">
-        <f aca="false">IF(AND(B26=Inputs!$C$28,H26&lt;&gt;"",L26&lt;&gt;"",H26&gt;=HMB!$C$53*(1+Inputs!$C$51),L26&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B26=Inputs!$C$28,H26&lt;&gt;"",L26&lt;&gt;"",D26&gt;=Inputs!$C$52,H26&gt;=HMB!$C$53*(1+Inputs!$C$51),L26&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N26" s="68" t="n">
@@ -10101,7 +10121,7 @@
       <c r="O26" s="70"/>
       <c r="P26" s="71"/>
       <c r="Q26" s="16" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10109,7 +10129,7 @@
         <v>99</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D27" s="72"/>
       <c r="E27" s="72"/>
@@ -10122,7 +10142,7 @@
         <v/>
       </c>
       <c r="H27" s="73" t="str">
-        <f aca="false">IF(F27="","",F27*Inputs!$C$44*Inputs!$C$53)</f>
+        <f aca="false">IF(F27="","",F27*Inputs!$C$44*Inputs!$C$54)</f>
         <v/>
       </c>
       <c r="I27" s="27"/>
@@ -10139,7 +10159,7 @@
         <v/>
       </c>
       <c r="M27" s="69" t="n">
-        <f aca="false">IF(AND(B27=Inputs!$C$28,H27&lt;&gt;"",L27&lt;&gt;"",H27&gt;=HMB!$C$53*(1+Inputs!$C$51),L27&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B27=Inputs!$C$28,H27&lt;&gt;"",L27&lt;&gt;"",D27&gt;=Inputs!$C$52,H27&gt;=HMB!$C$53*(1+Inputs!$C$51),L27&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N27" s="68" t="str">
@@ -10149,7 +10169,7 @@
       <c r="O27" s="70"/>
       <c r="P27" s="71"/>
       <c r="Q27" s="16" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10157,7 +10177,7 @@
         <v>102</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D28" s="17" t="n">
         <v>6</v>
@@ -10190,7 +10210,7 @@
         <v>5428.67210540316</v>
       </c>
       <c r="M28" s="69" t="n">
-        <f aca="false">IF(AND(B28=Inputs!$C$28,H28&lt;&gt;"",L28&lt;&gt;"",H28&gt;=HMB!$C$53*(1+Inputs!$C$51),L28&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B28=Inputs!$C$28,H28&lt;&gt;"",L28&lt;&gt;"",D28&gt;=Inputs!$C$52,H28&gt;=HMB!$C$53*(1+Inputs!$C$51),L28&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N28" s="68" t="n">
@@ -10200,7 +10220,7 @@
       <c r="O28" s="70"/>
       <c r="P28" s="71"/>
       <c r="Q28" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10208,7 +10228,7 @@
         <v>102</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D29" s="17" t="n">
         <v>8</v>
@@ -10241,7 +10261,7 @@
         <v>14074.3350880823</v>
       </c>
       <c r="M29" s="69" t="n">
-        <f aca="false">IF(AND(B29=Inputs!$C$28,H29&lt;&gt;"",L29&lt;&gt;"",H29&gt;=HMB!$C$53*(1+Inputs!$C$51),L29&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B29=Inputs!$C$28,H29&lt;&gt;"",L29&lt;&gt;"",D29&gt;=Inputs!$C$52,H29&gt;=HMB!$C$53*(1+Inputs!$C$51),L29&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N29" s="68" t="n">
@@ -10251,7 +10271,7 @@
       <c r="O29" s="70"/>
       <c r="P29" s="71"/>
       <c r="Q29" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10259,7 +10279,7 @@
         <v>102</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D30" s="17" t="n">
         <v>10</v>
@@ -10292,7 +10312,7 @@
         <v>25132.7412287183</v>
       </c>
       <c r="M30" s="69" t="n">
-        <f aca="false">IF(AND(B30=Inputs!$C$28,H30&lt;&gt;"",L30&lt;&gt;"",H30&gt;=HMB!$C$53*(1+Inputs!$C$51),L30&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B30=Inputs!$C$28,H30&lt;&gt;"",L30&lt;&gt;"",D30&gt;=Inputs!$C$52,H30&gt;=HMB!$C$53*(1+Inputs!$C$51),L30&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N30" s="68" t="n">
@@ -10302,7 +10322,7 @@
       <c r="O30" s="70"/>
       <c r="P30" s="71"/>
       <c r="Q30" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10310,7 +10330,7 @@
         <v>102</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D31" s="17" t="n">
         <v>10</v>
@@ -10343,7 +10363,7 @@
         <v>31415.9265358979</v>
       </c>
       <c r="M31" s="69" t="n">
-        <f aca="false">IF(AND(B31=Inputs!$C$28,H31&lt;&gt;"",L31&lt;&gt;"",H31&gt;=HMB!$C$53*(1+Inputs!$C$51),L31&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B31=Inputs!$C$28,H31&lt;&gt;"",L31&lt;&gt;"",D31&gt;=Inputs!$C$52,H31&gt;=HMB!$C$53*(1+Inputs!$C$51),L31&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N31" s="68" t="n">
@@ -10353,7 +10373,7 @@
       <c r="O31" s="70"/>
       <c r="P31" s="71"/>
       <c r="Q31" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10361,7 +10381,7 @@
         <v>102</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="D32" s="17" t="n">
         <v>12</v>
@@ -10394,7 +10414,7 @@
         <v>45238.934211693</v>
       </c>
       <c r="M32" s="69" t="n">
-        <f aca="false">IF(AND(B32=Inputs!$C$28,H32&lt;&gt;"",L32&lt;&gt;"",H32&gt;=HMB!$C$53*(1+Inputs!$C$51),L32&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B32=Inputs!$C$28,H32&lt;&gt;"",L32&lt;&gt;"",D32&gt;=Inputs!$C$52,H32&gt;=HMB!$C$53*(1+Inputs!$C$51),L32&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N32" s="68" t="n">
@@ -10404,7 +10424,7 @@
       <c r="O32" s="70"/>
       <c r="P32" s="71"/>
       <c r="Q32" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10412,7 +10432,7 @@
         <v>102</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D33" s="17" t="n">
         <v>12</v>
@@ -10445,7 +10465,7 @@
         <v>54286.7210540316</v>
       </c>
       <c r="M33" s="69" t="n">
-        <f aca="false">IF(AND(B33=Inputs!$C$28,H33&lt;&gt;"",L33&lt;&gt;"",H33&gt;=HMB!$C$53*(1+Inputs!$C$51),L33&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B33=Inputs!$C$28,H33&lt;&gt;"",L33&lt;&gt;"",D33&gt;=Inputs!$C$52,H33&gt;=HMB!$C$53*(1+Inputs!$C$51),L33&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N33" s="68" t="n">
@@ -10455,7 +10475,7 @@
       <c r="O33" s="70"/>
       <c r="P33" s="71"/>
       <c r="Q33" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10463,7 +10483,7 @@
         <v>102</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="D34" s="17" t="n">
         <v>12</v>
@@ -10496,7 +10516,7 @@
         <v>63334.5078963702</v>
       </c>
       <c r="M34" s="69" t="n">
-        <f aca="false">IF(AND(B34=Inputs!$C$28,H34&lt;&gt;"",L34&lt;&gt;"",H34&gt;=HMB!$C$53*(1+Inputs!$C$51),L34&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B34=Inputs!$C$28,H34&lt;&gt;"",L34&lt;&gt;"",D34&gt;=Inputs!$C$52,H34&gt;=HMB!$C$53*(1+Inputs!$C$51),L34&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N34" s="68" t="n">
@@ -10506,7 +10526,7 @@
       <c r="O34" s="70"/>
       <c r="P34" s="71"/>
       <c r="Q34" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10514,7 +10534,7 @@
         <v>102</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D35" s="17" t="n">
         <v>13</v>
@@ -10547,7 +10567,7 @@
         <v>63711.499014801</v>
       </c>
       <c r="M35" s="69" t="n">
-        <f aca="false">IF(AND(B35=Inputs!$C$28,H35&lt;&gt;"",L35&lt;&gt;"",H35&gt;=HMB!$C$53*(1+Inputs!$C$51),L35&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B35=Inputs!$C$28,H35&lt;&gt;"",L35&lt;&gt;"",D35&gt;=Inputs!$C$52,H35&gt;=HMB!$C$53*(1+Inputs!$C$51),L35&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N35" s="68" t="n">
@@ -10557,7 +10577,7 @@
       <c r="O35" s="70"/>
       <c r="P35" s="71"/>
       <c r="Q35" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10565,7 +10585,7 @@
         <v>102</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="D36" s="17" t="n">
         <v>14</v>
@@ -10598,7 +10618,7 @@
         <v>86205.3024145039</v>
       </c>
       <c r="M36" s="69" t="n">
-        <f aca="false">IF(AND(B36=Inputs!$C$28,H36&lt;&gt;"",L36&lt;&gt;"",H36&gt;=HMB!$C$53*(1+Inputs!$C$51),L36&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B36=Inputs!$C$28,H36&lt;&gt;"",L36&lt;&gt;"",D36&gt;=Inputs!$C$52,H36&gt;=HMB!$C$53*(1+Inputs!$C$51),L36&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N36" s="68" t="n">
@@ -10608,7 +10628,7 @@
       <c r="O36" s="70"/>
       <c r="P36" s="71"/>
       <c r="Q36" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10616,7 +10636,7 @@
         <v>102</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="D37" s="17" t="n">
         <v>15</v>
@@ -10649,7 +10669,7 @@
         <v>98960.1685880785</v>
       </c>
       <c r="M37" s="69" t="n">
-        <f aca="false">IF(AND(B37=Inputs!$C$28,H37&lt;&gt;"",L37&lt;&gt;"",H37&gt;=HMB!$C$53*(1+Inputs!$C$51),L37&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
+        <f aca="false">IF(AND(B37=Inputs!$C$28,H37&lt;&gt;"",L37&lt;&gt;"",D37&gt;=Inputs!$C$52,H37&gt;=HMB!$C$53*(1+Inputs!$C$51),L37&gt;=HMB!$C$9*(1+Inputs!$C$51)),ROW(),99999)</f>
         <v>99999</v>
       </c>
       <c r="N37" s="68" t="n">
@@ -10659,7 +10679,7 @@
       <c r="O37" s="70"/>
       <c r="P37" s="71"/>
       <c r="Q37" s="16" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
   </sheetData>
@@ -10690,7 +10710,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10703,7 +10723,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="10" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="C4" s="59" t="str">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$C$6:$C$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0)),"NO MODEL OF THIS TYPE MEETS THE JOB - fill ratings or pick another type")</f>
@@ -10725,7 +10745,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C6" s="60" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$E$6:$E$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0)),"")</f>
@@ -10737,19 +10757,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C7" s="29" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$G$6:$G$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0)),0)</f>
         <v>490.873852123405</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="C8" s="29" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$H$6:$H$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0)),"")</f>
@@ -10761,7 +10781,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C9" s="29" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$L$6:$L$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0)),"")</f>
@@ -10773,7 +10793,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="C10" s="60" t="str">
         <f aca="false">IFERROR(IF(INDEX('Dryer Models'!$I$6:$I$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0))="","not entered",INDEX('Dryer Models'!$I$6:$I$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0))),"")</f>
@@ -10785,7 +10805,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C11" s="60" t="n">
         <f aca="false">IFERROR(INDEX('Dryer Models'!$N$6:$N$37,MATCH(MIN('Dryer Models'!$M$6:$M$37),'Dryer Models'!$M$6:$M$37,0)),"")</f>
@@ -10795,12 +10815,12 @@
         <v>41</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="10" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">HMB!$C$80</f>
@@ -10822,7 +10842,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C14" s="30" t="n">
         <f aca="false">IF(ISNUMBER(Equipment!$C$9),HMB!$C$9/Equipment!$C$9,"")</f>
@@ -10832,7 +10852,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -10840,7 +10860,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C16" s="11" t="n">
         <f aca="false">HMB!$C$29/1000000</f>
@@ -10852,7 +10872,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="10" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C17" s="65" t="n">
         <f aca="false">Equipment!$C$16*(1+Inputs!$C$50)</f>
@@ -10864,7 +10884,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C18" s="29" t="str">
         <f aca="false">IF(AND(ISNUMBER(Equipment!$C$10),Equipment!$C$10&gt;0),IF(Equipment!$C$17&lt;=Equipment!$C$10,"WITHIN MODEL BURNER RATING","EXCEEDS MODEL BURNER RATING - next size or bigger burner"),"model burner rating not entered")</f>
@@ -10874,46 +10894,46 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C19" s="29" t="n">
-        <f aca="false">Equipment!$C$17*1000000/Inputs!$C$52</f>
+        <f aca="false">Equipment!$C$17*1000000/Inputs!$C$53</f>
         <v>2333.33333333333</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>64</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C20" s="60" t="n">
         <f aca="false">Equipment!$C$19/576</f>
         <v>4.05092592592593</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C21" s="60" t="n">
         <f aca="false">Equipment!$C$19/135</f>
         <v>17.283950617284</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C22" s="29" t="n">
         <f aca="false">ROUNDUP(Equipment!$C$17*100,-1)</f>
@@ -10921,12 +10941,12 @@
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="16" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
@@ -10934,7 +10954,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">HMB!$C$53</f>
@@ -10946,7 +10966,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="8" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C25" s="9" t="n">
         <f aca="false">Inputs!$C$38</f>
@@ -10958,37 +10978,37 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C26" s="60" t="n">
         <f aca="false">Equipment!$C$24*Inputs!$C$45/(6356*Inputs!$C$46)</f>
         <v>9.41405727562118</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="10" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="C27" s="59" t="n">
         <f aca="false">INDEX(Tables!$B$4:$B$21,COUNTIF(Tables!$B$4:$B$21,"&lt;"&amp;Equipment!$C$26*1.15)+1)</f>
         <v>15</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="C28" s="60" t="n">
         <f aca="false">SQRT(Equipment!$C$24/Inputs!$C$47*4/PI())*12</f>
@@ -11000,7 +11020,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="10" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C29" s="59" t="n">
         <f aca="false">CEILING(Equipment!$C$28,2)</f>
@@ -11012,7 +11032,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C30" s="29" t="n">
         <f aca="false">Equipment!$C$24/(PI()/4*(Equipment!$C$29/12)^2)</f>
@@ -11024,7 +11044,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="8" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="C31" s="29" t="n">
         <f aca="false">CEILING(SQRT(HMB!$C$60/Inputs!$C$47*4/PI())*12,2)</f>
@@ -11036,7 +11056,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="8" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C32" s="29" t="n">
         <f aca="false">Equipment!$C$24/Inputs!$C$48*144</f>
@@ -11046,12 +11066,12 @@
         <v>64</v>
       </c>
       <c r="E32" s="16" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="8" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C33" s="29" t="n">
         <f aca="false">SQRT(Equipment!$C$24/Inputs!$C$48/0.125)*12</f>
@@ -11061,12 +11081,12 @@
         <v>69</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="6" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
@@ -11074,31 +11094,31 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="8" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">HMB!$C$7/Inputs!$C$19/60</f>
         <v>3.47222222222222</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">Inputs!$C$13/Inputs!$C$20/60</f>
         <v>4.16666666666667</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="10" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="C37" s="59" t="n">
         <f aca="false">IFERROR(INDEX(Tables!$E$4:$E$13,COUNTIF(Tables!$H$4:$H$13,"&lt;"&amp;Equipment!$C$35)+1),"none in table")</f>
@@ -11108,7 +11128,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="10" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C38" s="59" t="n">
         <f aca="false">IFERROR(INDEX(Tables!$E$4:$E$13,COUNTIF(Tables!$H$4:$H$13,"&lt;"&amp;Equipment!$C$36)+1),"none in table")</f>
@@ -11118,7 +11138,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C39" s="29" t="n">
         <f aca="false">IFERROR(INDEX(Tables!$J$4:$J$13,COUNTIF(Tables!$M$4:$M$13,"&lt;"&amp;Equipment!$C$36*60)+1),"none in table")</f>
@@ -11141,7 +11161,7 @@
         <v>74</v>
       </c>
       <c r="C41" s="9" t="n">
-        <f aca="false">Inputs!$C$59</f>
+        <f aca="false">Inputs!$C$60</f>
         <v>7488</v>
       </c>
       <c r="D41" s="8" t="s">
@@ -11162,7 +11182,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="C43" s="29" t="n">
         <f aca="false">HMB!$C$9*Equipment!$C$41/2000</f>
@@ -11210,7 +11230,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="10" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="C47" s="75" t="n">
         <f aca="false">IF(Equipment!$C$42&gt;0,Equipment!$C$46/Equipment!$C$42,0)</f>
@@ -11254,39 +11274,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="10" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="I3" s="20" t="s">
+        <v>468</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>469</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>470</v>
+      </c>
+      <c r="L3" s="20" t="s">
         <v>466</v>
       </c>
-      <c r="J3" s="20" t="s">
-        <v>467</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>468</v>
-      </c>
-      <c r="L3" s="20" t="s">
-        <v>464</v>
-      </c>
       <c r="M3" s="20" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11604,10 +11624,10 @@
         <v>75</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="J14" s="16" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11675,12 +11695,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="4" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="6" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -11691,77 +11711,77 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="8" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="C4" s="26" t="n">
         <v>0.1</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="8" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="C5" s="26" t="n">
         <v>0.08</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="H5" s="16" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="8" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="C6" s="78" t="n">
         <v>0.0006</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="H6" s="16" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="8" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>0.9</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="8" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>3</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="8" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="C9" s="25" t="n">
         <v>0.9</v>
@@ -11770,12 +11790,12 @@
         <v>169</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="8" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="C10" s="25" t="n">
         <v>0.7</v>
@@ -11784,12 +11804,12 @@
         <v>169</v>
       </c>
       <c r="H10" s="16" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C11" s="25" t="n">
         <v>0.15</v>
@@ -11798,12 +11818,12 @@
         <v>169</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -11814,34 +11834,34 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="20" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C13" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="C14" s="79" t="n">
         <f aca="false">HMB!$C$31*Inputs!$C$35</f>
         <v>281.432748538012</v>
       </c>
       <c r="D14" s="79" t="n">
-        <f aca="false">C14*Inputs!$C$59/2000</f>
+        <f aca="false">C14*Inputs!$C$60/2000</f>
         <v>1053.68421052632</v>
       </c>
       <c r="E14" s="79" t="n">
@@ -11859,14 +11879,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="C15" s="79" t="n">
         <f aca="false">HMB!$C$29/1000000*Emissions!$C$4</f>
         <v>0.233333333333333</v>
       </c>
       <c r="D15" s="79" t="n">
-        <f aca="false">C15*Inputs!$C$59/2000</f>
+        <f aca="false">C15*Inputs!$C$60/2000</f>
         <v>0.8736</v>
       </c>
       <c r="E15" s="79" t="n">
@@ -11884,14 +11904,14 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="C16" s="79" t="n">
         <f aca="false">HMB!$C$29/1000000*Emissions!$C$5</f>
         <v>0.186666666666667</v>
       </c>
       <c r="D16" s="79" t="n">
-        <f aca="false">C16*Inputs!$C$59/2000</f>
+        <f aca="false">C16*Inputs!$C$60/2000</f>
         <v>0.69888</v>
       </c>
       <c r="E16" s="79" t="n">
@@ -11909,14 +11929,14 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C17" s="79" t="n">
         <f aca="false">HMB!$C$29/1000000*Emissions!$C$6</f>
         <v>0.0014</v>
       </c>
       <c r="D17" s="79" t="n">
-        <f aca="false">C17*Inputs!$C$59/2000</f>
+        <f aca="false">C17*Inputs!$C$60/2000</f>
         <v>0.0052416</v>
       </c>
       <c r="E17" s="79" t="n">
@@ -11934,14 +11954,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="C18" s="79" t="n">
         <f aca="false">Emissions!$C$7*(HMB!$C$5/2000)</f>
         <v>0.675</v>
       </c>
       <c r="D18" s="79" t="n">
-        <f aca="false">C18*Inputs!$C$59/2000</f>
+        <f aca="false">C18*Inputs!$C$60/2000</f>
         <v>2.5272</v>
       </c>
       <c r="E18" s="79" t="n">
@@ -11959,14 +11979,14 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="C19" s="79" t="n">
         <f aca="false">Emissions!$C$11*Emissions!$C$7*(HMB!$C$5/2000)</f>
         <v>0.10125</v>
       </c>
       <c r="D19" s="79" t="n">
-        <f aca="false">C19*Inputs!$C$59/2000</f>
+        <f aca="false">C19*Inputs!$C$60/2000</f>
         <v>0.37908</v>
       </c>
       <c r="E19" s="79" t="n">
@@ -11984,14 +12004,14 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C20" s="79" t="n">
         <f aca="false">Emissions!$C$8*(HMB!$C$5/2000)*(1-Emissions!$C$9)</f>
         <v>0.225</v>
       </c>
       <c r="D20" s="79" t="n">
-        <f aca="false">C20*Inputs!$C$59/2000</f>
+        <f aca="false">C20*Inputs!$C$60/2000</f>
         <v>0.8424</v>
       </c>
       <c r="E20" s="79" t="n">
@@ -12009,14 +12029,14 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="C21" s="79" t="n">
         <f aca="false">Emissions!$C$8*(HMB!$C$5/2000)*(1-Emissions!$C$9)*Emissions!$C$10</f>
         <v>0.1575</v>
       </c>
       <c r="D21" s="79" t="n">
-        <f aca="false">C21*Inputs!$C$59/2000</f>
+        <f aca="false">C21*Inputs!$C$60/2000</f>
         <v>0.58968</v>
       </c>
       <c r="E21" s="79" t="n">

</xml_diff>